<commit_message>
Improve Infinity Forge prompt variety
</commit_message>
<xml_diff>
--- a/Infinity_Forge_Prompts_Master.xlsx
+++ b/Infinity_Forge_Prompts_Master.xlsx
@@ -401,2502 +401,2502 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>A horned demon hero appears with black obsidian armor with ember seams. stands guard with one arm outstretched as if holding back a riot. The scene is set in a rain-slick alley lined with broken neon, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A horned guardian enters from the smoke with a amber lantern as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>A glamorous demon queen appears with curved horns, violet eyes, and a jeweled corset of armor. stands with one hip angled, half invitation and half warning. The scene is set in a cathedral chamber lit by purple fire, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. stands with one hip angled, half invitation and half warning.</v>
+        <v>A glamorous demon queen poses without apology with a amber crown as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>A cosmic tyrant appears with a crown of broken rings and black armor that drinks in starlight. hovers above the scene like a sentence already carried out. The scene is set in a broken ring world, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. hovers above the scene like a sentence already carried out.</v>
+        <v>A cosmic tyrant floats above the wreckage with a amber dagger as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>A spiky-haired martial artist appears with an orange training suit and a bright electric aura. holds a stance that feels like the start of a new transformation. The scene is set in an arena floor split by shockwaves, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. holds a stance that feels like the start of a new transformation.</v>
+        <v>A spiky-haired fighter surges into the shot with a amber banner as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>A transforming robot knight appears with silver armor panels and blue optics. stands mid-transformation while plates shift and locks release. The scene is set in a launch bay full of warning lights, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. stands mid-transformation while plates shift and locks release.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a amber compass as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>A hell-born guardian appears with a torn cape over scarred stone skin. turns at three-quarters view while sparks climb the armor. The scene is set in a collapsed overpass above a flooded street, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. plants a sword into the pavement like a promise.</v>
+        <v>A pale swordswoman stands in the rain with a amber mirror as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>A succubus antihero appears with translucent wings and clawed gloves. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a black marble throne room, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. balances a weapon with theatrical ease.</v>
+        <v>A barbarian champion charges forward with a amber sigil as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>A void emperor appears with purple lightning crawling over heavy metal plates. stands perfectly still while debris orbits around him. The scene is set in the edge of a collapsing black hole, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. extends both arms as if pulling planets into place.</v>
+        <v>A wizard opens a glowing spellbook with a amber helm as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>A supercharged fighter appears with silver hair, a torn gi, and sparks on the shoulders. raises both hands in disciplined preparation for a special move. The scene is set in a mountain plateau under electric clouds, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. leans forward, ready to cross the distance in one breath.</v>
+        <v>A final fusion champion stands in impossible balance with a amber orb as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>A chrome battle guardian appears with visible transformation seams and a reactor chest. kneels briefly as if receiving a command sequence. The scene is set in a ruined highway overpass, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A demon-born rescuer plants his feet with a amber chain as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>A volcanic avenger appears with heavy gauntlets and a glowing chest sigil. leans into the wind as if the whole skyline is listening. The scene is set in a courthouse roof beneath a bruised sunset, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A horned enchantress steps into the frame with a amber blade as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>A horned battle sorceress appears with polished white plating with bright blue optics. holds still in a pose that feels expensive and lethal. The scene is set in a rooftop garden under a blood moon, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A void emperor commands the frame with a amber pouch as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>A star-eating monarch appears with a cape shaped like a collapsing nebula. raises a hand and makes the horizon feel smaller. The scene is set in a dead moon covered in ice cliffs, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. looks down at the world with pitiless patience.</v>
+        <v>A power-charged martial artist braces for impact with a amber ring as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>A gravity-breaking warrior appears with a clenched fist surrounded by white light. keeps his chin high as the aura swells around him. The scene is set in a desert plain with shattered pillars, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. smiles briefly before tightening back into focus.</v>
+        <v>A chrome battle guardian shifts into combat form with a amber torch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>A vehicle-shaped mech hero appears with blocky legs and sleek forearms. braces in a landing pose with dust kicking outward. The scene is set in a smoke-filled hangar, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A scarred hunter moves through the ruins with a amber tablet as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>A bat-winged vigilante appears with winged shoulder plates and clawed gloves. holds position with the stillness of a veteran. The scene is set in a subway platform split by glowing cracks, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. leans into the wind as if the whole skyline is listening.</v>
+        <v>A fur-clad warrior bellows in the open air with a amber key as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>A chrome guardian heroine appears with a cockpit-like chest core and heavy machine joints. stands poised like a queen deciding who may live. The scene is set in a foggy canal lined with lanterns, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. holds still in a pose that feels expensive and lethal.</v>
+        <v>A battle mage lifts a hand and the air bends with a amber mask as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>A dimensional conqueror appears with a mask hiding every trace of mercy. carries the stillness of a final boss before the last phase. The scene is set in a starship graveyard, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. raises a hand and makes the horizon feel smaller.</v>
+        <v>An ultimate crossover hero fills the frame with a amber idol as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>A disciplined combat prodigy appears with boots planted wide on broken stone. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a battlefield of smoke and broken stone, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. keeps his chin high as the aura swells around him.</v>
+        <v>A hell-forged vigilante turns toward the street with a amber chalice as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>A towering machine duelist appears with wing-like shoulder fins and bright thrusters. locks into a battle form that looks ready for the final charge. The scene is set in a city street cracked by artillery fire, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. braces in a landing pose with dust kicking outward.</v>
+        <v>A seductive antihero turns to face the viewer with a amber quartz as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>A red-skinned protector appears with a cracked helmet and blazing eyes. plants a sword into the pavement like a promise. The scene is set in a plaza of shattered statues and smoke, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. freezes for a beat before launching into motion.</v>
+        <v>A star-eating monarch watches in silence with a crimson lantern as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>A machine-bodied temptress appears with smoke-colored hair and floating ember jewelry. balances a weapon with theatrical ease. The scene is set in a shattered ballroom with broken chandeliers, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. turns just enough to show both beauty and threat.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a crimson crown as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>A black-hole despot appears with gravity ripples bending around the shoulders. extends both arms as if pulling planets into place. The scene is set in a cathedral of empty space, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. walks forward through the void as though space is a corridor.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a crimson dagger as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>A tournament legend appears with a face that stays calm for only a second. leans forward, ready to cross the distance in one breath. The scene is set in a cliff edge above a storm sea, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A grim blade carrier watches the tree line with a crimson banner as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>A future war protector appears with a visor that opens like a cockpit canopy. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a moonbase platform under floodlights, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. spreads wing panels before taking off.</v>
+        <v>A savage axe fighter sets his stance with a crimson compass as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>A cursed city sentinel appears with a broad chest wrapped in iron bands. raises a fist to summon flame around the knuckles. The scene is set in a firelit dockyard full of black water, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A spellcaster stands inside a circle of runes with a crimson mirror as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>A neon succubus pilot appears with a fitted bodysuit traced with circuit-like runes. tilts her chin up as if challenging the viewer directly. The scene is set in a hangar full of red warning lights, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. stands with one hip angled, half invitation and half warning.</v>
+        <v>A hybrid ruler of monsters and machines appears with a crimson sigil as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>A comet warlord appears with an obsidian throne strapped to the back like a relic. turns slightly as if the entire sky belongs to him. The scene is set in a shattered asteroid throne hall, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. hovers above the scene like a sentence already carried out.</v>
+        <v>A black-winged defender walks into the light with a crimson helm as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>A blue-flame brawler appears with a blue energy blaze rolling off the body. settles into a low posture that promises a violent burst of speed. The scene is set in a ruined training hall, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. holds a stance that feels like the start of a new transformation.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a crimson orb as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>A jet-form sentinel appears with mechanical plating ready to fold into another mode. opens a chest panel to reveal a glowing core. The scene is set in a drydock beside a stormy sea, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. stands mid-transformation while plates shift and locks release.</v>
+        <v>A galaxy breaker rises from the dark with a crimson chain as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>A smoke-wreathed champion appears with charcoal armor lit by molten cracks. freezes for a beat before launching into motion. The scene is set in a narrow canyon of apartment towers, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. plants a sword into the pavement like a promise.</v>
+        <v>A tournament legend gathers force in silence with a crimson blade as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>A black-winged war queen appears with a regal collar and black lacquered shoulder armor. turns just enough to show both beauty and threat. The scene is set in a neon alley reflecting rain on the pavement, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. balances a weapon with theatrical ease.</v>
+        <v>A towering machine duelist reconfigures its armor with a crimson pouch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>A galaxy breaker appears with glowing runes orbiting a towering silhouette. walks forward through the void as though space is a corridor. The scene is set in a nebula storm full of lightning, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. extends both arms as if pulling planets into place.</v>
+        <v>A battle-worn slayer pauses at the gate with a crimson ring as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>A sky-shattering combatant appears with a sleeveless uniform shredded by battle. crouches as if the whole battle is a spring wound too tight. The scene is set in a forest clearing with torn banners, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. leans forward, ready to cross the distance in one breath.</v>
+        <v>A tribal hero raises a weapon overhead with a crimson torch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>A tank-born champion appears with a sword mounted along the forearm. spreads wing panels before taking off. The scene is set in a maintenance tunnel under a fortress, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A scholarly mage turns toward the storm with a crimson tablet as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>A fire-eyed rescuer appears with a battle belt full of charms and relics. steps forward through ash without breaking eye contact. The scene is set in a ruined chapel with torn banners, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A mythic defender forged from every genre takes shape with a crimson key as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>A retro robot defender appears with chunky retro panels in primary colors. spreads her wings as though she owns the air around her. The scene is set in a moonlit bridge over dark water, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>An ember-eyed avenger breaks through the haze with a crimson mask as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>An astral usurper appears with hands wrapped in crackling violet energy. rests one hand on a throne made of shattered moons. The scene is set in a ruined observatory on a distant planet, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. looks down at the world with pitiless patience.</v>
+        <v>A moonlit temptress stands with dangerous grace with a crimson idol as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>A dragon-aura hero appears with a focused stare and wind whipping the hair upward. stands after impact as if the hit only sharpened his resolve. The scene is set in a rooftop under a violet lightning storm, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. smiles briefly before tightening back into focus.</v>
+        <v>A dimensional conqueror bends the sky with a crimson chalice as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>A stealth mech defender appears with heavy shoulders shaped with anime clarity. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a shattered landing strip, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A blue-flame combatant looks ready to leap with a crimson quartz as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>A shadow-cloaked defender appears with a blade-hand forged from living fire. keeps a low ready stance, built for protecting civilians first. The scene is set in a glassy intersection after a meteor strike, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. leans into the wind as if the whole skyline is listening.</v>
+        <v>A future war protector drops from the sky with a cerulean lantern as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>A crimson inferno commander appears with a narrow waist and luminous mechanical limbs. keeps her hands relaxed even though the room feels dangerous. The scene is set in a crystal crypt under a low ceiling of smoke, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. holds still in a pose that feels expensive and lethal.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a cerulean crown as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>A moon-crowned ruler appears with a chest core shining like a dying star. looks down at the world with pitiless patience. The scene is set in a dark portal above a city, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. raises a hand and makes the horizon feel smaller.</v>
+        <v>A mountain-raised berserker crouches low with a cerulean dagger as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>A hard-trained rival appears with a body built for speed and sudden impact. smiles briefly before tightening back into focus. The scene is set in a canyon lined with fallen statues, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. keeps his chin high as the aura swells around him.</v>
+        <v>An arcane prodigy gathers light between the fingers with a cerulean banner as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>A winged machine paladin appears with a body built from clean angular geometry. launches forward with sparks and motion blur trailing behind. The scene is set in a rusted factory floor, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. braces in a landing pose with dust kicking outward.</v>
+        <v>A last-boss guardian steps into the center of the scene with a cerulean compass as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>A crater-born hero appears with a cloak stitched from soot-colored cloth. looks over one shoulder, alert for a second attack. The scene is set in a stairway descending into red fog, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. freezes for a beat before launching into motion.</v>
+        <v>A horned guardian enters from the smoke with a cerulean mirror as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>A sleek armored enchantress appears with a faceplate that opens into a calm human stare. lets sparks drift from her fingers without looking down. The scene is set in a vault of ancient machine parts, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. turns just enough to show both beauty and threat.</v>
+        <v>A glamorous demon queen poses without apology with a cerulean sigil as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>A universe-devouring sovereign appears with armor plated with sharp comet-like fins. waits without expression, which makes the threat worse. The scene is set in a field of fragments from lost civilizations, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. walks forward through the void as though space is a corridor.</v>
+        <v>A cosmic tyrant floats above the wreckage with a cerulean helm as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>A power-surged champion appears with gloves wrapped in crackling energy bands. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a circular pit scarred by repeated battles, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A spiky-haired fighter surges into the shot with a cerulean orb as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>A battle android guardian appears with warning lights blinking across the torso. turns the head just enough to suggest a human presence inside. The scene is set in a rooftop docking station, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. spreads wing panels before taking off.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a cerulean chain as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>A horned demon hero appears with a torn cape over scarred stone skin. steps forward through ash without breaking eye contact. The scene is set in a courthouse roof beneath a bruised sunset, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. steps forward through ash without breaking eye contact.</v>
+        <v>A pale swordswoman stands in the rain with a cerulean blade as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>A glamorous demon queen appears with translucent wings and clawed gloves. spreads her wings as though she owns the air around her. The scene is set in a rooftop garden under a blood moon, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. spreads her wings as though she owns the air around her.</v>
+        <v>A barbarian champion charges forward with a cerulean pouch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>A cosmic tyrant appears with purple lightning crawling over heavy metal plates. rests one hand on a throne made of shattered moons. The scene is set in a dead moon covered in ice cliffs, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. rests one hand on a throne made of shattered moons.</v>
+        <v>A wizard opens a glowing spellbook with a cerulean ring as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>A spiky-haired martial artist appears with silver hair, a torn gi, and sparks on the shoulders. stands after impact as if the hit only sharpened his resolve. The scene is set in a desert plain with shattered pillars, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A final fusion champion stands in impossible balance with a cerulean torch as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>A transforming robot knight appears with visible transformation seams and a reactor chest. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a smoke-filled hangar, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A demon-born rescuer plants his feet with a cerulean tablet as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>A hell-born guardian appears with heavy gauntlets and a glowing chest sigil. keeps a low ready stance, built for protecting civilians first. The scene is set in a subway platform split by glowing cracks, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A horned enchantress steps into the frame with a cerulean key as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>A succubus antihero appears with polished white plating with bright blue optics. keeps her hands relaxed even though the room feels dangerous. The scene is set in a foggy canal lined with lanterns, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A void emperor commands the frame with a cerulean mask as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>A void emperor appears with a cape shaped like a collapsing nebula. looks down at the world with pitiless patience. The scene is set in a starship graveyard, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. stands perfectly still while debris orbits around him.</v>
+        <v>A power-charged martial artist braces for impact with a cerulean idol as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>A supercharged fighter appears with a clenched fist surrounded by white light. smiles briefly before tightening back into focus. The scene is set in a battlefield of smoke and broken stone, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. raises both hands in disciplined preparation for a special move.</v>
+        <v>A chrome battle guardian shifts into combat form with a cerulean chalice as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>A chrome battle guardian appears with blocky legs and sleek forearms. launches forward with sparks and motion blur trailing behind. The scene is set in a city street cracked by artillery fire, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. kneels briefly as if receiving a command sequence.</v>
+        <v>A scarred hunter moves through the ruins with a cerulean quartz as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>A volcanic avenger appears with winged shoulder plates and clawed gloves. looks over one shoulder, alert for a second attack. The scene is set in a plaza of shattered statues and smoke, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. raises a fist to summon flame around the knuckles.</v>
+        <v>A fur-clad warrior bellows in the open air with a ashen lantern as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>A horned battle sorceress appears with a cockpit-like chest core and heavy machine joints. lets sparks drift from her fingers without looking down. The scene is set in a shattered ballroom with broken chandeliers, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A battle mage lifts a hand and the air bends with a ashen crown as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>A star-eating monarch appears with a mask hiding every trace of mercy. waits without expression, which makes the threat worse. The scene is set in a cathedral of empty space, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. turns slightly as if the entire sky belongs to him.</v>
+        <v>An ultimate crossover hero fills the frame with a ashen dagger as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>A gravity-breaking warrior appears with boots planted wide on broken stone. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a cliff edge above a storm sea, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A hell-forged vigilante turns toward the street with a ashen banner as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>A vehicle-shaped mech hero appears with wing-like shoulder fins and bright thrusters. turns the head just enough to suggest a human presence inside. The scene is set in a moonbase platform under floodlights, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. opens a chest panel to reveal a glowing core.</v>
+        <v>A seductive antihero turns to face the viewer with a ashen compass as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>A bat-winged vigilante appears with a cracked helmet and blazing eyes. stands guard with one arm outstretched as if holding back a riot. The scene is set in a firelit dockyard full of black water, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. looks over one shoulder, alert for a second attack.</v>
+        <v>A star-eating monarch watches in silence with a ashen mirror as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>A chrome guardian heroine appears with smoke-colored hair and floating ember jewelry. stands with one hip angled, half invitation and half warning. The scene is set in a hangar full of red warning lights, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. lets sparks drift from her fingers without looking down.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a ashen sigil as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>A dimensional conqueror appears with gravity ripples bending around the shoulders. hovers above the scene like a sentence already carried out. The scene is set in a shattered asteroid throne hall, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. waits without expression, which makes the threat worse.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a ashen helm as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>A disciplined combat prodigy appears with a face that stays calm for only a second. holds a stance that feels like the start of a new transformation. The scene is set in a ruined training hall, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A grim blade carrier watches the tree line with a ashen orb as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>A towering machine duelist appears with a visor that opens like a cockpit canopy. stands mid-transformation while plates shift and locks release. The scene is set in a drydock beside a stormy sea, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. turns the head just enough to suggest a human presence inside.</v>
+        <v>A savage axe fighter sets his stance with a ashen chain as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>A red-skinned protector appears with a broad chest wrapped in iron bands. turns at three-quarters view while sparks climb the armor. The scene is set in a narrow canyon of apartment towers, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. holds position with the stillness of a veteran.</v>
+        <v>A spellcaster stands inside a circle of runes with a ashen blade as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>A machine-bodied temptress appears with a fitted bodysuit traced with circuit-like runes. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a neon alley reflecting rain on the pavement, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. stands poised like a queen deciding who may live.</v>
+        <v>A hybrid ruler of monsters and machines appears with a ashen pouch as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>A black-hole despot appears with an obsidian throne strapped to the back like a relic. stands perfectly still while debris orbits around him. The scene is set in a nebula storm full of lightning, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. carries the stillness of a final boss before the last phase.</v>
+        <v>A black-winged defender walks into the light with a ashen ring as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>A tournament legend appears with a blue energy blaze rolling off the body. raises both hands in disciplined preparation for a special move. The scene is set in a forest clearing with torn banners, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a ashen torch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>A future war protector appears with mechanical plating ready to fold into another mode. kneels briefly as if receiving a command sequence. The scene is set in a maintenance tunnel under a fortress, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. locks into a battle form that looks ready for the final charge.</v>
+        <v>A galaxy breaker rises from the dark with a ashen tablet as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>A cursed city sentinel appears with charcoal armor lit by molten cracks. leans into the wind as if the whole skyline is listening. The scene is set in a ruined chapel with torn banners, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. steps forward through ash without breaking eye contact.</v>
+        <v>A tournament legend gathers force in silence with a ashen key as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>A neon succubus pilot appears with a regal collar and black lacquered shoulder armor. holds still in a pose that feels expensive and lethal. The scene is set in a moonlit bridge over dark water, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. spreads her wings as though she owns the air around her.</v>
+        <v>A towering machine duelist reconfigures its armor with a ashen mask as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>A comet warlord appears with glowing runes orbiting a towering silhouette. raises a hand and makes the horizon feel smaller. The scene is set in a ruined observatory on a distant planet, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. rests one hand on a throne made of shattered moons.</v>
+        <v>A battle-worn slayer pauses at the gate with a ashen idol as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>A blue-flame brawler appears with a sleeveless uniform shredded by battle. keeps his chin high as the aura swells around him. The scene is set in a rooftop under a violet lightning storm, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A tribal hero raises a weapon overhead with a ashen chalice as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>A jet-form sentinel appears with a sword mounted along the forearm. braces in a landing pose with dust kicking outward. The scene is set in a shattered landing strip, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A scholarly mage turns toward the storm with a ashen quartz as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>A smoke-wreathed champion appears with a battle belt full of charms and relics. holds position with the stillness of a veteran. The scene is set in a glassy intersection after a meteor strike, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A mythic defender forged from every genre takes shape with a emerald lantern as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>A black-winged war queen appears with chunky retro panels in primary colors. stands poised like a queen deciding who may live. The scene is set in a crystal crypt under a low ceiling of smoke, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>An ember-eyed avenger breaks through the haze with a emerald crown as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>A galaxy breaker appears with hands wrapped in crackling violet energy. carries the stillness of a final boss before the last phase. The scene is set in a dark portal above a city, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. stands perfectly still while debris orbits around him.</v>
+        <v>A moonlit temptress stands with dangerous grace with a emerald dagger as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>A sky-shattering combatant appears with a focused stare and wind whipping the hair upward. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a canyon lined with fallen statues, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. raises both hands in disciplined preparation for a special move.</v>
+        <v>A dimensional conqueror bends the sky with a emerald banner as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>A tank-born champion appears with heavy shoulders shaped with anime clarity. locks into a battle form that looks ready for the final charge. The scene is set in a rusted factory floor, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. kneels briefly as if receiving a command sequence.</v>
+        <v>A blue-flame combatant looks ready to leap with a emerald compass as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>A fire-eyed rescuer appears with a blade-hand forged from living fire. plants a sword into the pavement like a promise. The scene is set in a stairway descending into red fog, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. raises a fist to summon flame around the knuckles.</v>
+        <v>A future war protector drops from the sky with a emerald mirror as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>A retro robot defender appears with a narrow waist and luminous mechanical limbs. balances a weapon with theatrical ease. The scene is set in a vault of ancient machine parts, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a emerald sigil as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>An astral usurper appears with a chest core shining like a dying star. extends both arms as if pulling planets into place. The scene is set in a field of fragments from lost civilizations, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. turns slightly as if the entire sky belongs to him.</v>
+        <v>A mountain-raised berserker crouches low with a emerald helm as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>A dragon-aura hero appears with a body built for speed and sudden impact. leans forward, ready to cross the distance in one breath. The scene is set in a circular pit scarred by repeated battles, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. settles into a low posture that promises a violent burst of speed.</v>
+        <v>An arcane prodigy gathers light between the fingers with a emerald orb as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>A stealth mech defender appears with a body built from clean angular geometry. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a rooftop docking station, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. opens a chest panel to reveal a glowing core.</v>
+        <v>A last-boss guardian steps into the center of the scene with a emerald chain as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>A shadow-cloaked defender appears with a cloak stitched from soot-colored cloth. raises a fist to summon flame around the knuckles. The scene is set in a rain-slick alley lined with broken neon, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. looks over one shoulder, alert for a second attack.</v>
+        <v>A horned guardian enters from the smoke with a emerald blade as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>A crimson inferno commander appears with a faceplate that opens into a calm human stare. tilts her chin up as if challenging the viewer directly. The scene is set in a cathedral chamber lit by purple fire, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. lets sparks drift from her fingers without looking down.</v>
+        <v>A glamorous demon queen poses without apology with a emerald pouch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>A moon-crowned ruler appears with armor plated with sharp comet-like fins. turns slightly as if the entire sky belongs to him. The scene is set in a broken ring world, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. waits without expression, which makes the threat worse.</v>
+        <v>A cosmic tyrant floats above the wreckage with a emerald ring as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>A hard-trained rival appears with gloves wrapped in crackling energy bands. settles into a low posture that promises a violent burst of speed. The scene is set in an arena floor split by shockwaves, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A spiky-haired fighter surges into the shot with a emerald torch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>A winged machine paladin appears with warning lights blinking across the torso. opens a chest panel to reveal a glowing core. The scene is set in a launch bay full of warning lights, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. turns the head just enough to suggest a human presence inside.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a emerald tablet as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>A crater-born hero appears with black obsidian armor with ember seams. freezes for a beat before launching into motion. The scene is set in a collapsed overpass above a flooded street, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. holds position with the stillness of a veteran.</v>
+        <v>A pale swordswoman stands in the rain with a emerald key as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>A sleek armored enchantress appears with curved horns, violet eyes, and a jeweled corset of armor. turns just enough to show both beauty and threat. The scene is set in a black marble throne room, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. stands poised like a queen deciding who may live.</v>
+        <v>A barbarian champion charges forward with a emerald mask as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>A universe-devouring sovereign appears with a crown of broken rings and black armor that drinks in starlight. walks forward through the void as though space is a corridor. The scene is set in the edge of a collapsing black hole, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. carries the stillness of a final boss before the last phase.</v>
+        <v>A wizard opens a glowing spellbook with a emerald idol as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>A power-surged champion appears with an orange training suit and a bright electric aura. crouches as if the whole battle is a spring wound too tight. The scene is set in a mountain plateau under electric clouds, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A final fusion champion stands in impossible balance with a emerald chalice as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>A battle android guardian appears with silver armor panels and blue optics. spreads wing panels before taking off. The scene is set in a ruined highway overpass, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. locks into a battle form that looks ready for the final charge.</v>
+        <v>A demon-born rescuer plants his feet with a emerald quartz as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>A horned demon hero appears with heavy gauntlets and a glowing chest sigil. plants a sword into the pavement like a promise. The scene is set in a plaza of shattered statues and smoke, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. plants a sword into the pavement like a promise.</v>
+        <v>A horned enchantress steps into the frame with a violet lantern as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>A glamorous demon queen appears with polished white plating with bright blue optics. balances a weapon with theatrical ease. The scene is set in a shattered ballroom with broken chandeliers, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. balances a weapon with theatrical ease.</v>
+        <v>A void emperor commands the frame with a violet crown as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>A cosmic tyrant appears with a cape shaped like a collapsing nebula. extends both arms as if pulling planets into place. The scene is set in a cathedral of empty space, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. extends both arms as if pulling planets into place.</v>
+        <v>A power-charged martial artist braces for impact with a violet dagger as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>A spiky-haired martial artist appears with a clenched fist surrounded by white light. leans forward, ready to cross the distance in one breath. The scene is set in a cliff edge above a storm sea, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. leans forward, ready to cross the distance in one breath.</v>
+        <v>A chrome battle guardian shifts into combat form with a violet banner as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>A transforming robot knight appears with blocky legs and sleek forearms. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a moonbase platform under floodlights, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A scarred hunter moves through the ruins with a violet compass as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>A hell-born guardian appears with winged shoulder plates and clawed gloves. raises a fist to summon flame around the knuckles. The scene is set in a firelit dockyard full of black water, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A fur-clad warrior bellows in the open air with a violet mirror as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>A succubus antihero appears with a cockpit-like chest core and heavy machine joints. tilts her chin up as if challenging the viewer directly. The scene is set in a hangar full of red warning lights, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A battle mage lifts a hand and the air bends with a violet sigil as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>A void emperor appears with a mask hiding every trace of mercy. turns slightly as if the entire sky belongs to him. The scene is set in a shattered asteroid throne hall, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. looks down at the world with pitiless patience.</v>
+        <v>An ultimate crossover hero fills the frame with a violet helm as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>A supercharged fighter appears with boots planted wide on broken stone. settles into a low posture that promises a violent burst of speed. The scene is set in a ruined training hall, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. smiles briefly before tightening back into focus.</v>
+        <v>A hell-forged vigilante turns toward the street with a violet orb as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>A chrome battle guardian appears with wing-like shoulder fins and bright thrusters. opens a chest panel to reveal a glowing core. The scene is set in a drydock beside a stormy sea, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A seductive antihero turns to face the viewer with a violet chain as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>A volcanic avenger appears with a cracked helmet and blazing eyes. freezes for a beat before launching into motion. The scene is set in a narrow canyon of apartment towers, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. leans into the wind as if the whole skyline is listening.</v>
+        <v>A star-eating monarch watches in silence with a violet blade as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>A horned battle sorceress appears with smoke-colored hair and floating ember jewelry. turns just enough to show both beauty and threat. The scene is set in a neon alley reflecting rain on the pavement, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. holds still in a pose that feels expensive and lethal.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a violet pouch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>A star-eating monarch appears with gravity ripples bending around the shoulders. walks forward through the void as though space is a corridor. The scene is set in a nebula storm full of lightning, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. raises a hand and makes the horizon feel smaller.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a violet ring as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>A gravity-breaking warrior appears with a face that stays calm for only a second. crouches as if the whole battle is a spring wound too tight. The scene is set in a forest clearing with torn banners, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. keeps his chin high as the aura swells around him.</v>
+        <v>A grim blade carrier watches the tree line with a violet torch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>A vehicle-shaped mech hero appears with a visor that opens like a cockpit canopy. spreads wing panels before taking off. The scene is set in a maintenance tunnel under a fortress, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. braces in a landing pose with dust kicking outward.</v>
+        <v>A savage axe fighter sets his stance with a violet tablet as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>A bat-winged vigilante appears with a broad chest wrapped in iron bands. steps forward through ash without breaking eye contact. The scene is set in a ruined chapel with torn banners, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. freezes for a beat before launching into motion.</v>
+        <v>A spellcaster stands inside a circle of runes with a violet key as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>A chrome guardian heroine appears with a fitted bodysuit traced with circuit-like runes. spreads her wings as though she owns the air around her. The scene is set in a moonlit bridge over dark water, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. turns just enough to show both beauty and threat.</v>
+        <v>A hybrid ruler of monsters and machines appears with a violet mask as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>A dimensional conqueror appears with an obsidian throne strapped to the back like a relic. rests one hand on a throne made of shattered moons. The scene is set in a ruined observatory on a distant planet, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. walks forward through the void as though space is a corridor.</v>
+        <v>A black-winged defender walks into the light with a violet idol as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>A disciplined combat prodigy appears with a blue energy blaze rolling off the body. stands after impact as if the hit only sharpened his resolve. The scene is set in a rooftop under a violet lightning storm, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a violet chalice as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>A towering machine duelist appears with mechanical plating ready to fold into another mode. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a shattered landing strip, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. spreads wing panels before taking off.</v>
+        <v>A galaxy breaker rises from the dark with a violet quartz as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>A red-skinned protector appears with charcoal armor lit by molten cracks. keeps a low ready stance, built for protecting civilians first. The scene is set in a glassy intersection after a meteor strike, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A tournament legend gathers force in silence with a golden lantern as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>A machine-bodied temptress appears with a regal collar and black lacquered shoulder armor. keeps her hands relaxed even though the room feels dangerous. The scene is set in a crystal crypt under a low ceiling of smoke, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. stands with one hip angled, half invitation and half warning.</v>
+        <v>A towering machine duelist reconfigures its armor with a golden crown as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>A black-hole despot appears with glowing runes orbiting a towering silhouette. looks down at the world with pitiless patience. The scene is set in a dark portal above a city, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. hovers above the scene like a sentence already carried out.</v>
+        <v>A battle-worn slayer pauses at the gate with a golden dagger as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>A tournament legend appears with a sleeveless uniform shredded by battle. smiles briefly before tightening back into focus. The scene is set in a canyon lined with fallen statues, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. holds a stance that feels like the start of a new transformation.</v>
+        <v>A tribal hero raises a weapon overhead with a golden banner as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>A future war protector appears with a sword mounted along the forearm. launches forward with sparks and motion blur trailing behind. The scene is set in a rusted factory floor, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. stands mid-transformation while plates shift and locks release.</v>
+        <v>A scholarly mage turns toward the storm with a golden compass as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>A cursed city sentinel appears with a battle belt full of charms and relics. looks over one shoulder, alert for a second attack. The scene is set in a stairway descending into red fog, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. plants a sword into the pavement like a promise.</v>
+        <v>A mythic defender forged from every genre takes shape with a golden mirror as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>A neon succubus pilot appears with chunky retro panels in primary colors. lets sparks drift from her fingers without looking down. The scene is set in a vault of ancient machine parts, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. balances a weapon with theatrical ease.</v>
+        <v>An ember-eyed avenger breaks through the haze with a golden sigil as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>A comet warlord appears with hands wrapped in crackling violet energy. waits without expression, which makes the threat worse. The scene is set in a field of fragments from lost civilizations, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. extends both arms as if pulling planets into place.</v>
+        <v>A moonlit temptress stands with dangerous grace with a golden helm as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>A blue-flame brawler appears with a focused stare and wind whipping the hair upward. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a circular pit scarred by repeated battles, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. leans forward, ready to cross the distance in one breath.</v>
+        <v>A dimensional conqueror bends the sky with a golden orb as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>A jet-form sentinel appears with heavy shoulders shaped with anime clarity. turns the head just enough to suggest a human presence inside. The scene is set in a rooftop docking station, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A blue-flame combatant looks ready to leap with a golden chain as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>A smoke-wreathed champion appears with a blade-hand forged from living fire. stands guard with one arm outstretched as if holding back a riot. The scene is set in a rain-slick alley lined with broken neon, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A future war protector drops from the sky with a golden blade as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>A black-winged war queen appears with a narrow waist and luminous mechanical limbs. stands with one hip angled, half invitation and half warning. The scene is set in a cathedral chamber lit by purple fire, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a golden pouch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>A galaxy breaker appears with a chest core shining like a dying star. hovers above the scene like a sentence already carried out. The scene is set in a broken ring world, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. looks down at the world with pitiless patience.</v>
+        <v>A mountain-raised berserker crouches low with a golden ring as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>A sky-shattering combatant appears with a body built for speed and sudden impact. holds a stance that feels like the start of a new transformation. The scene is set in an arena floor split by shockwaves, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. smiles briefly before tightening back into focus.</v>
+        <v>An arcane prodigy gathers light between the fingers with a golden torch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>A tank-born champion appears with a body built from clean angular geometry. stands mid-transformation while plates shift and locks release. The scene is set in a launch bay full of warning lights, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A last-boss guardian steps into the center of the scene with a golden tablet as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>A fire-eyed rescuer appears with a cloak stitched from soot-colored cloth. turns at three-quarters view while sparks climb the armor. The scene is set in a collapsed overpass above a flooded street, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. leans into the wind as if the whole skyline is listening.</v>
+        <v>A horned guardian enters from the smoke with a golden key as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>A retro robot defender appears with a faceplate that opens into a calm human stare. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a black marble throne room, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. holds still in a pose that feels expensive and lethal.</v>
+        <v>A glamorous demon queen poses without apology with a golden mask as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>An astral usurper appears with armor plated with sharp comet-like fins. stands perfectly still while debris orbits around him. The scene is set in the edge of a collapsing black hole, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. raises a hand and makes the horizon feel smaller.</v>
+        <v>A cosmic tyrant floats above the wreckage with a golden idol as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>A dragon-aura hero appears with gloves wrapped in crackling energy bands. raises both hands in disciplined preparation for a special move. The scene is set in a mountain plateau under electric clouds, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. keeps his chin high as the aura swells around him.</v>
+        <v>A spiky-haired fighter surges into the shot with a golden chalice as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>A stealth mech defender appears with warning lights blinking across the torso. kneels briefly as if receiving a command sequence. The scene is set in a ruined highway overpass, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. braces in a landing pose with dust kicking outward.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a golden quartz as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>A shadow-cloaked defender appears with black obsidian armor with ember seams. leans into the wind as if the whole skyline is listening. The scene is set in a courthouse roof beneath a bruised sunset, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. freezes for a beat before launching into motion.</v>
+        <v>A pale swordswoman stands in the rain with a silver lantern as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>A crimson inferno commander appears with curved horns, violet eyes, and a jeweled corset of armor. holds still in a pose that feels expensive and lethal. The scene is set in a rooftop garden under a blood moon, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. turns just enough to show both beauty and threat.</v>
+        <v>A barbarian champion charges forward with a silver crown as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>A moon-crowned ruler appears with a crown of broken rings and black armor that drinks in starlight. raises a hand and makes the horizon feel smaller. The scene is set in a dead moon covered in ice cliffs, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. walks forward through the void as though space is a corridor.</v>
+        <v>A wizard opens a glowing spellbook with a silver dagger as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>A hard-trained rival appears with an orange training suit and a bright electric aura. keeps his chin high as the aura swells around him. The scene is set in a desert plain with shattered pillars, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A final fusion champion stands in impossible balance with a silver banner as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>A winged machine paladin appears with silver armor panels and blue optics. braces in a landing pose with dust kicking outward. The scene is set in a smoke-filled hangar, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. spreads wing panels before taking off.</v>
+        <v>A demon-born rescuer plants his feet with a silver compass as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>A crater-born hero appears with a torn cape over scarred stone skin. holds position with the stillness of a veteran. The scene is set in a subway platform split by glowing cracks, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A horned enchantress steps into the frame with a silver mirror as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>A sleek armored enchantress appears with translucent wings and clawed gloves. stands poised like a queen deciding who may live. The scene is set in a foggy canal lined with lanterns, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. stands with one hip angled, half invitation and half warning.</v>
+        <v>A void emperor commands the frame with a silver sigil as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>A universe-devouring sovereign appears with purple lightning crawling over heavy metal plates. carries the stillness of a final boss before the last phase. The scene is set in a starship graveyard, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. hovers above the scene like a sentence already carried out.</v>
+        <v>A power-charged martial artist braces for impact with a silver helm as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>A power-surged champion appears with silver hair, a torn gi, and sparks on the shoulders. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a battlefield of smoke and broken stone, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. holds a stance that feels like the start of a new transformation.</v>
+        <v>A chrome battle guardian shifts into combat form with a silver orb as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>A battle android guardian appears with visible transformation seams and a reactor chest. locks into a battle form that looks ready for the final charge. The scene is set in a city street cracked by artillery fire, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. stands mid-transformation while plates shift and locks release.</v>
+        <v>A scarred hunter moves through the ruins with a silver chain as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>A horned demon hero appears with winged shoulder plates and clawed gloves. turns at three-quarters view while sparks climb the armor. The scene is set in a narrow canyon of apartment towers, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A fur-clad warrior bellows in the open air with a silver blade as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>A glamorous demon queen appears with a cockpit-like chest core and heavy machine joints. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a neon alley reflecting rain on the pavement, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A battle mage lifts a hand and the air bends with a silver pouch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>A cosmic tyrant appears with a mask hiding every trace of mercy. stands perfectly still while debris orbits around him. The scene is set in a nebula storm full of lightning, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. stands perfectly still while debris orbits around him.</v>
+        <v>An ultimate crossover hero fills the frame with a silver ring as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>A spiky-haired martial artist appears with boots planted wide on broken stone. raises both hands in disciplined preparation for a special move. The scene is set in a forest clearing with torn banners, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. raises both hands in disciplined preparation for a special move.</v>
+        <v>A hell-forged vigilante turns toward the street with a silver torch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>A transforming robot knight appears with wing-like shoulder fins and bright thrusters. kneels briefly as if receiving a command sequence. The scene is set in a maintenance tunnel under a fortress, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. kneels briefly as if receiving a command sequence.</v>
+        <v>A seductive antihero turns to face the viewer with a silver tablet as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>A hell-born guardian appears with a cracked helmet and blazing eyes. leans into the wind as if the whole skyline is listening. The scene is set in a ruined chapel with torn banners, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. raises a fist to summon flame around the knuckles.</v>
+        <v>A star-eating monarch watches in silence with a silver key as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>A succubus antihero appears with smoke-colored hair and floating ember jewelry. holds still in a pose that feels expensive and lethal. The scene is set in a moonlit bridge over dark water, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a silver mask as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>A void emperor appears with gravity ripples bending around the shoulders. raises a hand and makes the horizon feel smaller. The scene is set in a ruined observatory on a distant planet, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. turns slightly as if the entire sky belongs to him.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a silver idol as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>A supercharged fighter appears with a face that stays calm for only a second. keeps his chin high as the aura swells around him. The scene is set in a rooftop under a violet lightning storm, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A grim blade carrier watches the tree line with a silver chalice as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>A chrome battle guardian appears with a visor that opens like a cockpit canopy. braces in a landing pose with dust kicking outward. The scene is set in a shattered landing strip, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. opens a chest panel to reveal a glowing core.</v>
+        <v>A savage axe fighter sets his stance with a silver quartz as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>A volcanic avenger appears with a broad chest wrapped in iron bands. holds position with the stillness of a veteran. The scene is set in a glassy intersection after a meteor strike, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. looks over one shoulder, alert for a second attack.</v>
+        <v>A spellcaster stands inside a circle of runes with a cobalt lantern as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>A horned battle sorceress appears with a fitted bodysuit traced with circuit-like runes. stands poised like a queen deciding who may live. The scene is set in a crystal crypt under a low ceiling of smoke, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. lets sparks drift from her fingers without looking down.</v>
+        <v>A hybrid ruler of monsters and machines appears with a cobalt crown as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>A star-eating monarch appears with an obsidian throne strapped to the back like a relic. carries the stillness of a final boss before the last phase. The scene is set in a dark portal above a city, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. waits without expression, which makes the threat worse.</v>
+        <v>A black-winged defender walks into the light with a cobalt dagger as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>A gravity-breaking warrior appears with a blue energy blaze rolling off the body. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a canyon lined with fallen statues, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a cobalt banner as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>A vehicle-shaped mech hero appears with mechanical plating ready to fold into another mode. locks into a battle form that looks ready for the final charge. The scene is set in a rusted factory floor, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. turns the head just enough to suggest a human presence inside.</v>
+        <v>A galaxy breaker rises from the dark with a cobalt compass as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>A bat-winged vigilante appears with charcoal armor lit by molten cracks. plants a sword into the pavement like a promise. The scene is set in a stairway descending into red fog, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. holds position with the stillness of a veteran.</v>
+        <v>A tournament legend gathers force in silence with a cobalt mirror as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>A chrome guardian heroine appears with a regal collar and black lacquered shoulder armor. balances a weapon with theatrical ease. The scene is set in a vault of ancient machine parts, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. stands poised like a queen deciding who may live.</v>
+        <v>A towering machine duelist reconfigures its armor with a cobalt sigil as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>A dimensional conqueror appears with glowing runes orbiting a towering silhouette. extends both arms as if pulling planets into place. The scene is set in a field of fragments from lost civilizations, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. carries the stillness of a final boss before the last phase.</v>
+        <v>A battle-worn slayer pauses at the gate with a cobalt helm as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>A disciplined combat prodigy appears with a sleeveless uniform shredded by battle. leans forward, ready to cross the distance in one breath. The scene is set in a circular pit scarred by repeated battles, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A tribal hero raises a weapon overhead with a cobalt orb as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>A towering machine duelist appears with a sword mounted along the forearm. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a rooftop docking station, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. locks into a battle form that looks ready for the final charge.</v>
+        <v>A scholarly mage turns toward the storm with a cobalt chain as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>A red-skinned protector appears with a battle belt full of charms and relics. raises a fist to summon flame around the knuckles. The scene is set in a rain-slick alley lined with broken neon, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. steps forward through ash without breaking eye contact.</v>
+        <v>A mythic defender forged from every genre takes shape with a cobalt blade as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>A machine-bodied temptress appears with chunky retro panels in primary colors. tilts her chin up as if challenging the viewer directly. The scene is set in a cathedral chamber lit by purple fire, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. spreads her wings as though she owns the air around her.</v>
+        <v>An ember-eyed avenger breaks through the haze with a cobalt pouch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>A black-hole despot appears with hands wrapped in crackling violet energy. turns slightly as if the entire sky belongs to him. The scene is set in a broken ring world, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. rests one hand on a throne made of shattered moons.</v>
+        <v>A moonlit temptress stands with dangerous grace with a cobalt ring as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>A tournament legend appears with a focused stare and wind whipping the hair upward. settles into a low posture that promises a violent burst of speed. The scene is set in an arena floor split by shockwaves, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A dimensional conqueror bends the sky with a cobalt torch as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>A future war protector appears with heavy shoulders shaped with anime clarity. opens a chest panel to reveal a glowing core. The scene is set in a launch bay full of warning lights, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A blue-flame combatant looks ready to leap with a cobalt tablet as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>A cursed city sentinel appears with a blade-hand forged from living fire. freezes for a beat before launching into motion. The scene is set in a collapsed overpass above a flooded street, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A future war protector drops from the sky with a cobalt key as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>A neon succubus pilot appears with a narrow waist and luminous mechanical limbs. turns just enough to show both beauty and threat. The scene is set in a black marble throne room, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a cobalt mask as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>A comet warlord appears with a chest core shining like a dying star. walks forward through the void as though space is a corridor. The scene is set in the edge of a collapsing black hole, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. stands perfectly still while debris orbits around him.</v>
+        <v>A mountain-raised berserker crouches low with a cobalt idol as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>A blue-flame brawler appears with a body built for speed and sudden impact. crouches as if the whole battle is a spring wound too tight. The scene is set in a mountain plateau under electric clouds, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. raises both hands in disciplined preparation for a special move.</v>
+        <v>An arcane prodigy gathers light between the fingers with a cobalt chalice as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>A jet-form sentinel appears with a body built from clean angular geometry. spreads wing panels before taking off. The scene is set in a ruined highway overpass, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. kneels briefly as if receiving a command sequence.</v>
+        <v>A last-boss guardian steps into the center of the scene with a cobalt quartz as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>A smoke-wreathed champion appears with a cloak stitched from soot-colored cloth. steps forward through ash without breaking eye contact. The scene is set in a courthouse roof beneath a bruised sunset, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. raises a fist to summon flame around the knuckles.</v>
+        <v>A horned guardian enters from the smoke with a obsidian lantern as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>A black-winged war queen appears with a faceplate that opens into a calm human stare. spreads her wings as though she owns the air around her. The scene is set in a rooftop garden under a blood moon, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A glamorous demon queen poses without apology with a obsidian crown as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>A galaxy breaker appears with armor plated with sharp comet-like fins. rests one hand on a throne made of shattered moons. The scene is set in a dead moon covered in ice cliffs, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. turns slightly as if the entire sky belongs to him.</v>
+        <v>A cosmic tyrant floats above the wreckage with a obsidian dagger as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>A sky-shattering combatant appears with gloves wrapped in crackling energy bands. stands after impact as if the hit only sharpened his resolve. The scene is set in a desert plain with shattered pillars, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A spiky-haired fighter surges into the shot with a obsidian banner as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>A tank-born champion appears with warning lights blinking across the torso. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a smoke-filled hangar, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. opens a chest panel to reveal a glowing core.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a obsidian compass as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>A fire-eyed rescuer appears with black obsidian armor with ember seams. keeps a low ready stance, built for protecting civilians first. The scene is set in a subway platform split by glowing cracks, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. looks over one shoulder, alert for a second attack.</v>
+        <v>A pale swordswoman stands in the rain with a obsidian mirror as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>A retro robot defender appears with curved horns, violet eyes, and a jeweled corset of armor. keeps her hands relaxed even though the room feels dangerous. The scene is set in a foggy canal lined with lanterns, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. lets sparks drift from her fingers without looking down.</v>
+        <v>A barbarian champion charges forward with a obsidian sigil as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>An astral usurper appears with a crown of broken rings and black armor that drinks in starlight. looks down at the world with pitiless patience. The scene is set in a starship graveyard, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. waits without expression, which makes the threat worse.</v>
+        <v>A wizard opens a glowing spellbook with a obsidian helm as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>A dragon-aura hero appears with an orange training suit and a bright electric aura. smiles briefly before tightening back into focus. The scene is set in a battlefield of smoke and broken stone, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A final fusion champion stands in impossible balance with a obsidian orb as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>A stealth mech defender appears with silver armor panels and blue optics. launches forward with sparks and motion blur trailing behind. The scene is set in a city street cracked by artillery fire, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. turns the head just enough to suggest a human presence inside.</v>
+        <v>A demon-born rescuer plants his feet with a obsidian chain as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>A shadow-cloaked defender appears with a torn cape over scarred stone skin. looks over one shoulder, alert for a second attack. The scene is set in a plaza of shattered statues and smoke, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. holds position with the stillness of a veteran.</v>
+        <v>A horned enchantress steps into the frame with a obsidian blade as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>A crimson inferno commander appears with translucent wings and clawed gloves. lets sparks drift from her fingers without looking down. The scene is set in a shattered ballroom with broken chandeliers, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. stands poised like a queen deciding who may live.</v>
+        <v>A void emperor commands the frame with a obsidian pouch as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>A moon-crowned ruler appears with purple lightning crawling over heavy metal plates. waits without expression, which makes the threat worse. The scene is set in a cathedral of empty space, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. carries the stillness of a final boss before the last phase.</v>
+        <v>A power-charged martial artist braces for impact with a obsidian ring as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>A hard-trained rival appears with silver hair, a torn gi, and sparks on the shoulders. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a cliff edge above a storm sea, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A chrome battle guardian shifts into combat form with a obsidian torch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>A winged machine paladin appears with visible transformation seams and a reactor chest. turns the head just enough to suggest a human presence inside. The scene is set in a moonbase platform under floodlights, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. locks into a battle form that looks ready for the final charge.</v>
+        <v>A scarred hunter moves through the ruins with a obsidian tablet as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>A crater-born hero appears with heavy gauntlets and a glowing chest sigil. stands guard with one arm outstretched as if holding back a riot. The scene is set in a firelit dockyard full of black water, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. steps forward through ash without breaking eye contact.</v>
+        <v>A fur-clad warrior bellows in the open air with a obsidian key as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>A sleek armored enchantress appears with polished white plating with bright blue optics. stands with one hip angled, half invitation and half warning. The scene is set in a hangar full of red warning lights, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. spreads her wings as though she owns the air around her.</v>
+        <v>A battle mage lifts a hand and the air bends with a obsidian mask as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>A universe-devouring sovereign appears with a cape shaped like a collapsing nebula. hovers above the scene like a sentence already carried out. The scene is set in a shattered asteroid throne hall, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. rests one hand on a throne made of shattered moons.</v>
+        <v>An ultimate crossover hero fills the frame with a obsidian idol as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>A power-surged champion appears with a clenched fist surrounded by white light. holds a stance that feels like the start of a new transformation. The scene is set in a ruined training hall, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A hell-forged vigilante turns toward the street with a obsidian chalice as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>A battle android guardian appears with blocky legs and sleek forearms. stands mid-transformation while plates shift and locks release. The scene is set in a drydock beside a stormy sea, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A seductive antihero turns to face the viewer with a obsidian quartz as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>A horned demon hero appears with a cracked helmet and blazing eyes. keeps a low ready stance, built for protecting civilians first. The scene is set in a glassy intersection after a meteor strike, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A star-eating monarch watches in silence with a ivory lantern as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>A glamorous demon queen appears with smoke-colored hair and floating ember jewelry. keeps her hands relaxed even though the room feels dangerous. The scene is set in a crystal crypt under a low ceiling of smoke, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a ivory crown as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>A cosmic tyrant appears with gravity ripples bending around the shoulders. looks down at the world with pitiless patience. The scene is set in a dark portal above a city, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. looks down at the world with pitiless patience.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a ivory dagger as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>A spiky-haired martial artist appears with a face that stays calm for only a second. smiles briefly before tightening back into focus. The scene is set in a canyon lined with fallen statues, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. smiles briefly before tightening back into focus.</v>
+        <v>A grim blade carrier watches the tree line with a ivory banner as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>A transforming robot knight appears with a visor that opens like a cockpit canopy. launches forward with sparks and motion blur trailing behind. The scene is set in a rusted factory floor, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A savage axe fighter sets his stance with a ivory compass as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>A hell-born guardian appears with a broad chest wrapped in iron bands. looks over one shoulder, alert for a second attack. The scene is set in a stairway descending into red fog, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. leans into the wind as if the whole skyline is listening.</v>
+        <v>A spellcaster stands inside a circle of runes with a ivory mirror as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>A succubus antihero appears with a fitted bodysuit traced with circuit-like runes. lets sparks drift from her fingers without looking down. The scene is set in a vault of ancient machine parts, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. holds still in a pose that feels expensive and lethal.</v>
+        <v>A hybrid ruler of monsters and machines appears with a ivory sigil as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>A void emperor appears with an obsidian throne strapped to the back like a relic. waits without expression, which makes the threat worse. The scene is set in a field of fragments from lost civilizations, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. raises a hand and makes the horizon feel smaller.</v>
+        <v>A black-winged defender walks into the light with a ivory helm as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>A supercharged fighter appears with a blue energy blaze rolling off the body. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a circular pit scarred by repeated battles, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. keeps his chin high as the aura swells around him.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a ivory orb as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>A chrome battle guardian appears with mechanical plating ready to fold into another mode. turns the head just enough to suggest a human presence inside. The scene is set in a rooftop docking station, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. braces in a landing pose with dust kicking outward.</v>
+        <v>A galaxy breaker rises from the dark with a ivory chain as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>A volcanic avenger appears with charcoal armor lit by molten cracks. stands guard with one arm outstretched as if holding back a riot. The scene is set in a rain-slick alley lined with broken neon, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. freezes for a beat before launching into motion.</v>
+        <v>A tournament legend gathers force in silence with a ivory blade as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>A horned battle sorceress appears with a regal collar and black lacquered shoulder armor. stands with one hip angled, half invitation and half warning. The scene is set in a cathedral chamber lit by purple fire, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. turns just enough to show both beauty and threat.</v>
+        <v>A towering machine duelist reconfigures its armor with a ivory pouch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>A star-eating monarch appears with glowing runes orbiting a towering silhouette. hovers above the scene like a sentence already carried out. The scene is set in a broken ring world, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. walks forward through the void as though space is a corridor.</v>
+        <v>A battle-worn slayer pauses at the gate with a ivory ring as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>A gravity-breaking warrior appears with a sleeveless uniform shredded by battle. holds a stance that feels like the start of a new transformation. The scene is set in an arena floor split by shockwaves, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A tribal hero raises a weapon overhead with a ivory torch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>A vehicle-shaped mech hero appears with a sword mounted along the forearm. stands mid-transformation while plates shift and locks release. The scene is set in a launch bay full of warning lights, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. spreads wing panels before taking off.</v>
+        <v>A scholarly mage turns toward the storm with a ivory tablet as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>A bat-winged vigilante appears with a battle belt full of charms and relics. turns at three-quarters view while sparks climb the armor. The scene is set in a collapsed overpass above a flooded street, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A mythic defender forged from every genre takes shape with a ivory key as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>A chrome guardian heroine appears with chunky retro panels in primary colors. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a black marble throne room, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. stands with one hip angled, half invitation and half warning.</v>
+        <v>An ember-eyed avenger breaks through the haze with a ivory mask as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>A dimensional conqueror appears with hands wrapped in crackling violet energy. stands perfectly still while debris orbits around him. The scene is set in the edge of a collapsing black hole, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. hovers above the scene like a sentence already carried out.</v>
+        <v>A moonlit temptress stands with dangerous grace with a ivory idol as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>A disciplined combat prodigy appears with a focused stare and wind whipping the hair upward. raises both hands in disciplined preparation for a special move. The scene is set in a mountain plateau under electric clouds, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. holds a stance that feels like the start of a new transformation.</v>
+        <v>A dimensional conqueror bends the sky with a ivory chalice as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>A towering machine duelist appears with heavy shoulders shaped with anime clarity. kneels briefly as if receiving a command sequence. The scene is set in a ruined highway overpass, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. stands mid-transformation while plates shift and locks release.</v>
+        <v>A blue-flame combatant looks ready to leap with a ivory quartz as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>A red-skinned protector appears with a blade-hand forged from living fire. leans into the wind as if the whole skyline is listening. The scene is set in a courthouse roof beneath a bruised sunset, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. plants a sword into the pavement like a promise.</v>
+        <v>A future war protector drops from the sky with a scarlet lantern as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>A machine-bodied temptress appears with a narrow waist and luminous mechanical limbs. holds still in a pose that feels expensive and lethal. The scene is set in a rooftop garden under a blood moon, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. balances a weapon with theatrical ease.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a scarlet crown as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>A black-hole despot appears with a chest core shining like a dying star. raises a hand and makes the horizon feel smaller. The scene is set in a dead moon covered in ice cliffs, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. extends both arms as if pulling planets into place.</v>
+        <v>A mountain-raised berserker crouches low with a scarlet dagger as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>A tournament legend appears with a body built for speed and sudden impact. keeps his chin high as the aura swells around him. The scene is set in a desert plain with shattered pillars, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. leans forward, ready to cross the distance in one breath.</v>
+        <v>An arcane prodigy gathers light between the fingers with a scarlet banner as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>A future war protector appears with a body built from clean angular geometry. braces in a landing pose with dust kicking outward. The scene is set in a smoke-filled hangar, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A last-boss guardian steps into the center of the scene with a scarlet compass as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>A cursed city sentinel appears with a cloak stitched from soot-colored cloth. holds position with the stillness of a veteran. The scene is set in a subway platform split by glowing cracks, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A horned guardian enters from the smoke with a scarlet mirror as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>A neon succubus pilot appears with a faceplate that opens into a calm human stare. stands poised like a queen deciding who may live. The scene is set in a foggy canal lined with lanterns, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A glamorous demon queen poses without apology with a scarlet sigil as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>A comet warlord appears with armor plated with sharp comet-like fins. carries the stillness of a final boss before the last phase. The scene is set in a starship graveyard, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. looks down at the world with pitiless patience.</v>
+        <v>A cosmic tyrant floats above the wreckage with a scarlet helm as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>A blue-flame brawler appears with gloves wrapped in crackling energy bands. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a battlefield of smoke and broken stone, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. smiles briefly before tightening back into focus.</v>
+        <v>A spiky-haired fighter surges into the shot with a scarlet orb as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>A jet-form sentinel appears with warning lights blinking across the torso. locks into a battle form that looks ready for the final charge. The scene is set in a city street cracked by artillery fire, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a scarlet chain as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>A smoke-wreathed champion appears with black obsidian armor with ember seams. plants a sword into the pavement like a promise. The scene is set in a plaza of shattered statues and smoke, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. leans into the wind as if the whole skyline is listening.</v>
+        <v>A pale swordswoman stands in the rain with a scarlet blade as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>A black-winged war queen appears with curved horns, violet eyes, and a jeweled corset of armor. balances a weapon with theatrical ease. The scene is set in a shattered ballroom with broken chandeliers, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. holds still in a pose that feels expensive and lethal.</v>
+        <v>A barbarian champion charges forward with a scarlet pouch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>A galaxy breaker appears with a crown of broken rings and black armor that drinks in starlight. extends both arms as if pulling planets into place. The scene is set in a cathedral of empty space, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. raises a hand and makes the horizon feel smaller.</v>
+        <v>A wizard opens a glowing spellbook with a scarlet ring as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>A sky-shattering combatant appears with an orange training suit and a bright electric aura. leans forward, ready to cross the distance in one breath. The scene is set in a cliff edge above a storm sea, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. keeps his chin high as the aura swells around him.</v>
+        <v>A final fusion champion stands in impossible balance with a scarlet torch as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>A tank-born champion appears with silver armor panels and blue optics. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a moonbase platform under floodlights, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. braces in a landing pose with dust kicking outward.</v>
+        <v>A demon-born rescuer plants his feet with a scarlet tablet as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>A fire-eyed rescuer appears with a torn cape over scarred stone skin. raises a fist to summon flame around the knuckles. The scene is set in a firelit dockyard full of black water, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. freezes for a beat before launching into motion.</v>
+        <v>A horned enchantress steps into the frame with a scarlet key as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>A retro robot defender appears with translucent wings and clawed gloves. tilts her chin up as if challenging the viewer directly. The scene is set in a hangar full of red warning lights, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. turns just enough to show both beauty and threat.</v>
+        <v>A void emperor commands the frame with a scarlet mask as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>An astral usurper appears with purple lightning crawling over heavy metal plates. turns slightly as if the entire sky belongs to him. The scene is set in a shattered asteroid throne hall, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. walks forward through the void as though space is a corridor.</v>
+        <v>A power-charged martial artist braces for impact with a scarlet idol as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>A dragon-aura hero appears with silver hair, a torn gi, and sparks on the shoulders. settles into a low posture that promises a violent burst of speed. The scene is set in a ruined training hall, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A chrome battle guardian shifts into combat form with a scarlet chalice as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>A stealth mech defender appears with visible transformation seams and a reactor chest. opens a chest panel to reveal a glowing core. The scene is set in a drydock beside a stormy sea, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. spreads wing panels before taking off.</v>
+        <v>A scarred hunter moves through the ruins with a scarlet quartz as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>A shadow-cloaked defender appears with heavy gauntlets and a glowing chest sigil. freezes for a beat before launching into motion. The scene is set in a narrow canyon of apartment towers, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A fur-clad warrior bellows in the open air with a jade lantern as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>A crimson inferno commander appears with polished white plating with bright blue optics. turns just enough to show both beauty and threat. The scene is set in a neon alley reflecting rain on the pavement, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. stands with one hip angled, half invitation and half warning.</v>
+        <v>A battle mage lifts a hand and the air bends with a jade crown as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>A moon-crowned ruler appears with a cape shaped like a collapsing nebula. walks forward through the void as though space is a corridor. The scene is set in a nebula storm full of lightning, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. hovers above the scene like a sentence already carried out.</v>
+        <v>An ultimate crossover hero fills the frame with a jade dagger as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>A hard-trained rival appears with a clenched fist surrounded by white light. crouches as if the whole battle is a spring wound too tight. The scene is set in a forest clearing with torn banners, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. holds a stance that feels like the start of a new transformation.</v>
+        <v>A hell-forged vigilante turns toward the street with a jade banner as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>A winged machine paladin appears with blocky legs and sleek forearms. spreads wing panels before taking off. The scene is set in a maintenance tunnel under a fortress, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. stands mid-transformation while plates shift and locks release.</v>
+        <v>A seductive antihero turns to face the viewer with a jade compass as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>A crater-born hero appears with winged shoulder plates and clawed gloves. steps forward through ash without breaking eye contact. The scene is set in a ruined chapel with torn banners, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. plants a sword into the pavement like a promise.</v>
+        <v>A star-eating monarch watches in silence with a jade mirror as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>A sleek armored enchantress appears with a cockpit-like chest core and heavy machine joints. spreads her wings as though she owns the air around her. The scene is set in a moonlit bridge over dark water, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. balances a weapon with theatrical ease.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a jade sigil as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>A universe-devouring sovereign appears with a mask hiding every trace of mercy. rests one hand on a throne made of shattered moons. The scene is set in a ruined observatory on a distant planet, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. extends both arms as if pulling planets into place.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a jade helm as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>A power-surged champion appears with boots planted wide on broken stone. stands after impact as if the hit only sharpened his resolve. The scene is set in a rooftop under a violet lightning storm, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. leans forward, ready to cross the distance in one breath.</v>
+        <v>A grim blade carrier watches the tree line with a jade orb as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>A battle android guardian appears with wing-like shoulder fins and bright thrusters. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a shattered landing strip, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A savage axe fighter sets his stance with a jade chain as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>A horned demon hero appears with a broad chest wrapped in iron bands. raises a fist to summon flame around the knuckles. The scene is set in a rain-slick alley lined with broken neon, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. raises a fist to summon flame around the knuckles.</v>
+        <v>A spellcaster stands inside a circle of runes with a jade blade as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>A glamorous demon queen appears with a fitted bodysuit traced with circuit-like runes. tilts her chin up as if challenging the viewer directly. The scene is set in a cathedral chamber lit by purple fire, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A hybrid ruler of monsters and machines appears with a jade pouch as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>A cosmic tyrant appears with an obsidian throne strapped to the back like a relic. turns slightly as if the entire sky belongs to him. The scene is set in a broken ring world, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. turns slightly as if the entire sky belongs to him.</v>
+        <v>A black-winged defender walks into the light with a jade ring as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>A spiky-haired martial artist appears with a blue energy blaze rolling off the body. settles into a low posture that promises a violent burst of speed. The scene is set in an arena floor split by shockwaves, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a jade torch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>A transforming robot knight appears with mechanical plating ready to fold into another mode. opens a chest panel to reveal a glowing core. The scene is set in a launch bay full of warning lights, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. opens a chest panel to reveal a glowing core.</v>
+        <v>A galaxy breaker rises from the dark with a jade tablet as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>A hell-born guardian appears with charcoal armor lit by molten cracks. freezes for a beat before launching into motion. The scene is set in a collapsed overpass above a flooded street, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. looks over one shoulder, alert for a second attack.</v>
+        <v>A tournament legend gathers force in silence with a jade key as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>A succubus antihero appears with a regal collar and black lacquered shoulder armor. turns just enough to show both beauty and threat. The scene is set in a black marble throne room, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. lets sparks drift from her fingers without looking down.</v>
+        <v>A towering machine duelist reconfigures its armor with a jade mask as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>A void emperor appears with glowing runes orbiting a towering silhouette. walks forward through the void as though space is a corridor. The scene is set in the edge of a collapsing black hole, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. waits without expression, which makes the threat worse.</v>
+        <v>A battle-worn slayer pauses at the gate with a jade idol as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>A supercharged fighter appears with a sleeveless uniform shredded by battle. crouches as if the whole battle is a spring wound too tight. The scene is set in a mountain plateau under electric clouds, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A tribal hero raises a weapon overhead with a jade chalice as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>A chrome battle guardian appears with a sword mounted along the forearm. spreads wing panels before taking off. The scene is set in a ruined highway overpass, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. turns the head just enough to suggest a human presence inside.</v>
+        <v>A scholarly mage turns toward the storm with a jade quartz as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>A volcanic avenger appears with a battle belt full of charms and relics. steps forward through ash without breaking eye contact. The scene is set in a courthouse roof beneath a bruised sunset, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. holds position with the stillness of a veteran.</v>
+        <v>A mythic defender forged from every genre takes shape with a saffron lantern as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>A horned battle sorceress appears with chunky retro panels in primary colors. spreads her wings as though she owns the air around her. The scene is set in a rooftop garden under a blood moon, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. stands poised like a queen deciding who may live.</v>
+        <v>An ember-eyed avenger breaks through the haze with a saffron crown as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>A star-eating monarch appears with hands wrapped in crackling violet energy. rests one hand on a throne made of shattered moons. The scene is set in a dead moon covered in ice cliffs, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. carries the stillness of a final boss before the last phase.</v>
+        <v>A moonlit temptress stands with dangerous grace with a saffron dagger as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>A gravity-breaking warrior appears with a focused stare and wind whipping the hair upward. stands after impact as if the hit only sharpened his resolve. The scene is set in a desert plain with shattered pillars, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A dimensional conqueror bends the sky with a saffron banner as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>A vehicle-shaped mech hero appears with heavy shoulders shaped with anime clarity. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a smoke-filled hangar, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. locks into a battle form that looks ready for the final charge.</v>
+        <v>A blue-flame combatant looks ready to leap with a saffron compass as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>A bat-winged vigilante appears with a blade-hand forged from living fire. keeps a low ready stance, built for protecting civilians first. The scene is set in a subway platform split by glowing cracks, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. steps forward through ash without breaking eye contact.</v>
+        <v>A future war protector drops from the sky with a saffron mirror as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>A chrome guardian heroine appears with a narrow waist and luminous mechanical limbs. keeps her hands relaxed even though the room feels dangerous. The scene is set in a foggy canal lined with lanterns, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. spreads her wings as though she owns the air around her.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a saffron sigil as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>A dimensional conqueror appears with a chest core shining like a dying star. looks down at the world with pitiless patience. The scene is set in a starship graveyard, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. rests one hand on a throne made of shattered moons.</v>
+        <v>A mountain-raised berserker crouches low with a saffron helm as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>A disciplined combat prodigy appears with a body built for speed and sudden impact. smiles briefly before tightening back into focus. The scene is set in a battlefield of smoke and broken stone, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>An arcane prodigy gathers light between the fingers with a saffron orb as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>A towering machine duelist appears with a body built from clean angular geometry. launches forward with sparks and motion blur trailing behind. The scene is set in a city street cracked by artillery fire, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A last-boss guardian steps into the center of the scene with a saffron chain as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>A red-skinned protector appears with a cloak stitched from soot-colored cloth. looks over one shoulder, alert for a second attack. The scene is set in a plaza of shattered statues and smoke, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A horned guardian enters from the smoke with a saffron blade as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>A machine-bodied temptress appears with a faceplate that opens into a calm human stare. lets sparks drift from her fingers without looking down. The scene is set in a shattered ballroom with broken chandeliers, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A glamorous demon queen poses without apology with a saffron pouch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>A black-hole despot appears with armor plated with sharp comet-like fins. waits without expression, which makes the threat worse. The scene is set in a cathedral of empty space, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. stands perfectly still while debris orbits around him.</v>
+        <v>A cosmic tyrant floats above the wreckage with a saffron ring as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>A tournament legend appears with gloves wrapped in crackling energy bands. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a cliff edge above a storm sea, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. raises both hands in disciplined preparation for a special move.</v>
+        <v>A spiky-haired fighter surges into the shot with a saffron torch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>A future war protector appears with warning lights blinking across the torso. turns the head just enough to suggest a human presence inside. The scene is set in a moonbase platform under floodlights, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. kneels briefly as if receiving a command sequence.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a saffron tablet as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>A cursed city sentinel appears with black obsidian armor with ember seams. stands guard with one arm outstretched as if holding back a riot. The scene is set in a firelit dockyard full of black water, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. raises a fist to summon flame around the knuckles.</v>
+        <v>A pale swordswoman stands in the rain with a saffron key as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>A neon succubus pilot appears with curved horns, violet eyes, and a jeweled corset of armor. stands with one hip angled, half invitation and half warning. The scene is set in a hangar full of red warning lights, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A barbarian champion charges forward with a saffron mask as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>A comet warlord appears with a crown of broken rings and black armor that drinks in starlight. hovers above the scene like a sentence already carried out. The scene is set in a shattered asteroid throne hall, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. turns slightly as if the entire sky belongs to him.</v>
+        <v>A wizard opens a glowing spellbook with a saffron idol as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>A blue-flame brawler appears with an orange training suit and a bright electric aura. holds a stance that feels like the start of a new transformation. The scene is set in a ruined training hall, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A final fusion champion stands in impossible balance with a saffron chalice as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>A jet-form sentinel appears with silver armor panels and blue optics. stands mid-transformation while plates shift and locks release. The scene is set in a drydock beside a stormy sea, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. opens a chest panel to reveal a glowing core.</v>
+        <v>A demon-born rescuer plants his feet with a saffron quartz as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>A smoke-wreathed champion appears with a torn cape over scarred stone skin. turns at three-quarters view while sparks climb the armor. The scene is set in a narrow canyon of apartment towers, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. looks over one shoulder, alert for a second attack.</v>
+        <v>A horned enchantress steps into the frame with a pearl lantern as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>A black-winged war queen appears with translucent wings and clawed gloves. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a neon alley reflecting rain on the pavement, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. lets sparks drift from her fingers without looking down.</v>
+        <v>A void emperor commands the frame with a pearl crown as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>A galaxy breaker appears with purple lightning crawling over heavy metal plates. stands perfectly still while debris orbits around him. The scene is set in a nebula storm full of lightning, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. waits without expression, which makes the threat worse.</v>
+        <v>A power-charged martial artist braces for impact with a pearl dagger as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="str">
-        <v>A sky-shattering combatant appears with silver hair, a torn gi, and sparks on the shoulders. raises both hands in disciplined preparation for a special move. The scene is set in a forest clearing with torn banners, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A chrome battle guardian shifts into combat form with a pearl banner as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>A tank-born champion appears with visible transformation seams and a reactor chest. kneels briefly as if receiving a command sequence. The scene is set in a maintenance tunnel under a fortress, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. turns the head just enough to suggest a human presence inside.</v>
+        <v>A scarred hunter moves through the ruins with a pearl compass as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>A fire-eyed rescuer appears with heavy gauntlets and a glowing chest sigil. leans into the wind as if the whole skyline is listening. The scene is set in a ruined chapel with torn banners, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. holds position with the stillness of a veteran.</v>
+        <v>A fur-clad warrior bellows in the open air with a pearl mirror as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>A retro robot defender appears with polished white plating with bright blue optics. holds still in a pose that feels expensive and lethal. The scene is set in a moonlit bridge over dark water, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. stands poised like a queen deciding who may live.</v>
+        <v>A battle mage lifts a hand and the air bends with a pearl sigil as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>An astral usurper appears with a cape shaped like a collapsing nebula. raises a hand and makes the horizon feel smaller. The scene is set in a ruined observatory on a distant planet, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. carries the stillness of a final boss before the last phase.</v>
+        <v>An ultimate crossover hero fills the frame with a pearl helm as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>A dragon-aura hero appears with a clenched fist surrounded by white light. keeps his chin high as the aura swells around him. The scene is set in a rooftop under a violet lightning storm, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A hell-forged vigilante turns toward the street with a pearl orb as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>A stealth mech defender appears with blocky legs and sleek forearms. braces in a landing pose with dust kicking outward. The scene is set in a shattered landing strip, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. locks into a battle form that looks ready for the final charge.</v>
+        <v>A seductive antihero turns to face the viewer with a pearl chain as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>A shadow-cloaked defender appears with winged shoulder plates and clawed gloves. holds position with the stillness of a veteran. The scene is set in a glassy intersection after a meteor strike, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. steps forward through ash without breaking eye contact.</v>
+        <v>A star-eating monarch watches in silence with a pearl blade as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>A crimson inferno commander appears with a cockpit-like chest core and heavy machine joints. stands poised like a queen deciding who may live. The scene is set in a crystal crypt under a low ceiling of smoke, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. spreads her wings as though she owns the air around her.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a pearl pouch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>A moon-crowned ruler appears with a mask hiding every trace of mercy. carries the stillness of a final boss before the last phase. The scene is set in a dark portal above a city, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. rests one hand on a throne made of shattered moons.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a pearl ring as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>A hard-trained rival appears with boots planted wide on broken stone. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a canyon lined with fallen statues, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A grim blade carrier watches the tree line with a pearl torch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>A winged machine paladin appears with wing-like shoulder fins and bright thrusters. locks into a battle form that looks ready for the final charge. The scene is set in a rusted factory floor, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A savage axe fighter sets his stance with a pearl tablet as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>A crater-born hero appears with a cracked helmet and blazing eyes. plants a sword into the pavement like a promise. The scene is set in a stairway descending into red fog, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A spellcaster stands inside a circle of runes with a pearl key as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>A sleek armored enchantress appears with smoke-colored hair and floating ember jewelry. balances a weapon with theatrical ease. The scene is set in a vault of ancient machine parts, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A hybrid ruler of monsters and machines appears with a pearl mask as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>A universe-devouring sovereign appears with gravity ripples bending around the shoulders. extends both arms as if pulling planets into place. The scene is set in a field of fragments from lost civilizations, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. stands perfectly still while debris orbits around him.</v>
+        <v>A black-winged defender walks into the light with a pearl idol as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>A power-surged champion appears with a face that stays calm for only a second. leans forward, ready to cross the distance in one breath. The scene is set in a circular pit scarred by repeated battles, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. raises both hands in disciplined preparation for a special move.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a pearl chalice as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="str">
-        <v>A battle android guardian appears with a visor that opens like a cockpit canopy. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a rooftop docking station, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. kneels briefly as if receiving a command sequence.</v>
+        <v>A galaxy breaker rises from the dark with a pearl quartz as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="str">
-        <v>A horned demon hero appears with charcoal armor lit by molten cracks. leans into the wind as if the whole skyline is listening. The scene is set in a courthouse roof beneath a bruised sunset, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. leans into the wind as if the whole skyline is listening.</v>
+        <v>A tournament legend gathers force in silence with a onyx lantern as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>A glamorous demon queen appears with a regal collar and black lacquered shoulder armor. holds still in a pose that feels expensive and lethal. The scene is set in a rooftop garden under a blood moon, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. holds still in a pose that feels expensive and lethal.</v>
+        <v>A towering machine duelist reconfigures its armor with a onyx crown as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>A cosmic tyrant appears with glowing runes orbiting a towering silhouette. raises a hand and makes the horizon feel smaller. The scene is set in a dead moon covered in ice cliffs, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. raises a hand and makes the horizon feel smaller.</v>
+        <v>A battle-worn slayer pauses at the gate with a onyx dagger as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
-        <v>A spiky-haired martial artist appears with a sleeveless uniform shredded by battle. keeps his chin high as the aura swells around him. The scene is set in a desert plain with shattered pillars, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. keeps his chin high as the aura swells around him.</v>
+        <v>A tribal hero raises a weapon overhead with a onyx banner as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="str">
-        <v>A transforming robot knight appears with a sword mounted along the forearm. braces in a landing pose with dust kicking outward. The scene is set in a smoke-filled hangar, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. braces in a landing pose with dust kicking outward.</v>
+        <v>A scholarly mage turns toward the storm with a onyx compass as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="str">
-        <v>A hell-born guardian appears with a battle belt full of charms and relics. holds position with the stillness of a veteran. The scene is set in a subway platform split by glowing cracks, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. freezes for a beat before launching into motion.</v>
+        <v>A mythic defender forged from every genre takes shape with a onyx mirror as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>A succubus antihero appears with chunky retro panels in primary colors. stands poised like a queen deciding who may live. The scene is set in a foggy canal lined with lanterns, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. turns just enough to show both beauty and threat.</v>
+        <v>An ember-eyed avenger breaks through the haze with a onyx sigil as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>A void emperor appears with hands wrapped in crackling violet energy. carries the stillness of a final boss before the last phase. The scene is set in a starship graveyard, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. walks forward through the void as though space is a corridor.</v>
+        <v>A moonlit temptress stands with dangerous grace with a onyx helm as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>A supercharged fighter appears with a focused stare and wind whipping the hair upward. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a battlefield of smoke and broken stone, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A dimensional conqueror bends the sky with a onyx orb as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>A chrome battle guardian appears with heavy shoulders shaped with anime clarity. locks into a battle form that looks ready for the final charge. The scene is set in a city street cracked by artillery fire, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. spreads wing panels before taking off.</v>
+        <v>A blue-flame combatant looks ready to leap with a onyx chain as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>A volcanic avenger appears with a blade-hand forged from living fire. plants a sword into the pavement like a promise. The scene is set in a plaza of shattered statues and smoke, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A future war protector drops from the sky with a onyx blade as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>A horned battle sorceress appears with a narrow waist and luminous mechanical limbs. balances a weapon with theatrical ease. The scene is set in a shattered ballroom with broken chandeliers, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. stands with one hip angled, half invitation and half warning.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a onyx pouch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>A star-eating monarch appears with a chest core shining like a dying star. extends both arms as if pulling planets into place. The scene is set in a cathedral of empty space, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. hovers above the scene like a sentence already carried out.</v>
+        <v>A mountain-raised berserker crouches low with a onyx ring as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>A gravity-breaking warrior appears with a body built for speed and sudden impact. leans forward, ready to cross the distance in one breath. The scene is set in a cliff edge above a storm sea, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. holds a stance that feels like the start of a new transformation.</v>
+        <v>An arcane prodigy gathers light between the fingers with a onyx torch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>A vehicle-shaped mech hero appears with a body built from clean angular geometry. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a moonbase platform under floodlights, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. stands mid-transformation while plates shift and locks release.</v>
+        <v>A last-boss guardian steps into the center of the scene with a onyx tablet as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>A bat-winged vigilante appears with a cloak stitched from soot-colored cloth. raises a fist to summon flame around the knuckles. The scene is set in a firelit dockyard full of black water, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. plants a sword into the pavement like a promise.</v>
+        <v>A horned guardian enters from the smoke with a onyx key as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>A chrome guardian heroine appears with a faceplate that opens into a calm human stare. tilts her chin up as if challenging the viewer directly. The scene is set in a hangar full of red warning lights, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. balances a weapon with theatrical ease.</v>
+        <v>A glamorous demon queen poses without apology with a onyx mask as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>A dimensional conqueror appears with armor plated with sharp comet-like fins. turns slightly as if the entire sky belongs to him. The scene is set in a shattered asteroid throne hall, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. extends both arms as if pulling planets into place.</v>
+        <v>A cosmic tyrant floats above the wreckage with a onyx idol as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>A disciplined combat prodigy appears with gloves wrapped in crackling energy bands. settles into a low posture that promises a violent burst of speed. The scene is set in a ruined training hall, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. leans forward, ready to cross the distance in one breath.</v>
+        <v>A spiky-haired fighter surges into the shot with a onyx chalice as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>A towering machine duelist appears with warning lights blinking across the torso. opens a chest panel to reveal a glowing core. The scene is set in a drydock beside a stormy sea, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a onyx quartz as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
-        <v>A red-skinned protector appears with black obsidian armor with ember seams. freezes for a beat before launching into motion. The scene is set in a narrow canyon of apartment towers, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A pale swordswoman stands in the rain with a moss lantern as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="str">
-        <v>A machine-bodied temptress appears with curved horns, violet eyes, and a jeweled corset of armor. turns just enough to show both beauty and threat. The scene is set in a neon alley reflecting rain on the pavement, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A barbarian champion charges forward with a moss crown as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>A black-hole despot appears with a crown of broken rings and black armor that drinks in starlight. walks forward through the void as though space is a corridor. The scene is set in a nebula storm full of lightning, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. looks down at the world with pitiless patience.</v>
+        <v>A wizard opens a glowing spellbook with a moss dagger as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>A tournament legend appears with an orange training suit and a bright electric aura. crouches as if the whole battle is a spring wound too tight. The scene is set in a forest clearing with torn banners, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. smiles briefly before tightening back into focus.</v>
+        <v>A final fusion champion stands in impossible balance with a moss banner as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>A future war protector appears with silver armor panels and blue optics. spreads wing panels before taking off. The scene is set in a maintenance tunnel under a fortress, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A demon-born rescuer plants his feet with a moss compass as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="str">
-        <v>A cursed city sentinel appears with a torn cape over scarred stone skin. steps forward through ash without breaking eye contact. The scene is set in a ruined chapel with torn banners, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. leans into the wind as if the whole skyline is listening.</v>
+        <v>A horned enchantress steps into the frame with a moss mirror as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="str">
-        <v>A neon succubus pilot appears with translucent wings and clawed gloves. spreads her wings as though she owns the air around her. The scene is set in a moonlit bridge over dark water, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. holds still in a pose that feels expensive and lethal.</v>
+        <v>A void emperor commands the frame with a moss sigil as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="str">
-        <v>A comet warlord appears with purple lightning crawling over heavy metal plates. rests one hand on a throne made of shattered moons. The scene is set in a ruined observatory on a distant planet, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. raises a hand and makes the horizon feel smaller.</v>
+        <v>A power-charged martial artist braces for impact with a moss helm as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="str">
-        <v>A blue-flame brawler appears with silver hair, a torn gi, and sparks on the shoulders. stands after impact as if the hit only sharpened his resolve. The scene is set in a rooftop under a violet lightning storm, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. keeps his chin high as the aura swells around him.</v>
+        <v>A chrome battle guardian shifts into combat form with a moss orb as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="str">
-        <v>A jet-form sentinel appears with visible transformation seams and a reactor chest. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a shattered landing strip, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. braces in a landing pose with dust kicking outward.</v>
+        <v>A scarred hunter moves through the ruins with a moss chain as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>A smoke-wreathed champion appears with heavy gauntlets and a glowing chest sigil. keeps a low ready stance, built for protecting civilians first. The scene is set in a glassy intersection after a meteor strike, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. freezes for a beat before launching into motion.</v>
+        <v>A fur-clad warrior bellows in the open air with a moss blade as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>A black-winged war queen appears with polished white plating with bright blue optics. keeps her hands relaxed even though the room feels dangerous. The scene is set in a crystal crypt under a low ceiling of smoke, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. turns just enough to show both beauty and threat.</v>
+        <v>A battle mage lifts a hand and the air bends with a moss pouch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>A galaxy breaker appears with a cape shaped like a collapsing nebula. looks down at the world with pitiless patience. The scene is set in a dark portal above a city, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. walks forward through the void as though space is a corridor.</v>
+        <v>An ultimate crossover hero fills the frame with a moss ring as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>A sky-shattering combatant appears with a clenched fist surrounded by white light. smiles briefly before tightening back into focus. The scene is set in a canyon lined with fallen statues, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A hell-forged vigilante turns toward the street with a moss torch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>A tank-born champion appears with blocky legs and sleek forearms. launches forward with sparks and motion blur trailing behind. The scene is set in a rusted factory floor, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. spreads wing panels before taking off.</v>
+        <v>A seductive antihero turns to face the viewer with a moss tablet as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>A fire-eyed rescuer appears with winged shoulder plates and clawed gloves. looks over one shoulder, alert for a second attack. The scene is set in a stairway descending into red fog, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A star-eating monarch watches in silence with a moss key as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>A retro robot defender appears with a cockpit-like chest core and heavy machine joints. lets sparks drift from her fingers without looking down. The scene is set in a vault of ancient machine parts, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. stands with one hip angled, half invitation and half warning.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a moss mask as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>An astral usurper appears with a mask hiding every trace of mercy. waits without expression, which makes the threat worse. The scene is set in a field of fragments from lost civilizations, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. hovers above the scene like a sentence already carried out.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a moss idol as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>A dragon-aura hero appears with boots planted wide on broken stone. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a circular pit scarred by repeated battles, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. holds a stance that feels like the start of a new transformation.</v>
+        <v>A grim blade carrier watches the tree line with a moss chalice as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>A stealth mech defender appears with wing-like shoulder fins and bright thrusters. turns the head just enough to suggest a human presence inside. The scene is set in a rooftop docking station, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. stands mid-transformation while plates shift and locks release.</v>
+        <v>A savage axe fighter sets his stance with a moss quartz as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>A shadow-cloaked defender appears with a cracked helmet and blazing eyes. stands guard with one arm outstretched as if holding back a riot. The scene is set in a rain-slick alley lined with broken neon, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. plants a sword into the pavement like a promise.</v>
+        <v>A spellcaster stands inside a circle of runes with a ruby lantern as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>A crimson inferno commander appears with smoke-colored hair and floating ember jewelry. stands with one hip angled, half invitation and half warning. The scene is set in a cathedral chamber lit by purple fire, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. balances a weapon with theatrical ease.</v>
+        <v>A hybrid ruler of monsters and machines appears with a ruby crown as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>A moon-crowned ruler appears with gravity ripples bending around the shoulders. hovers above the scene like a sentence already carried out. The scene is set in a broken ring world, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. extends both arms as if pulling planets into place.</v>
+        <v>A black-winged defender walks into the light with a ruby dagger as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>A hard-trained rival appears with a face that stays calm for only a second. holds a stance that feels like the start of a new transformation. The scene is set in an arena floor split by shockwaves, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. leans forward, ready to cross the distance in one breath.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a ruby banner as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>A winged machine paladin appears with a visor that opens like a cockpit canopy. stands mid-transformation while plates shift and locks release. The scene is set in a launch bay full of warning lights, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A galaxy breaker rises from the dark with a ruby compass as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>A crater-born hero appears with a broad chest wrapped in iron bands. turns at three-quarters view while sparks climb the armor. The scene is set in a collapsed overpass above a flooded street, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A tournament legend gathers force in silence with a ruby mirror as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>A sleek armored enchantress appears with a fitted bodysuit traced with circuit-like runes. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a black marble throne room, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A towering machine duelist reconfigures its armor with a ruby sigil as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>A universe-devouring sovereign appears with an obsidian throne strapped to the back like a relic. stands perfectly still while debris orbits around him. The scene is set in the edge of a collapsing black hole, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. looks down at the world with pitiless patience.</v>
+        <v>A battle-worn slayer pauses at the gate with a ruby helm as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>A power-surged champion appears with a blue energy blaze rolling off the body. raises both hands in disciplined preparation for a special move. The scene is set in a mountain plateau under electric clouds, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. smiles briefly before tightening back into focus.</v>
+        <v>A tribal hero raises a weapon overhead with a ruby orb as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>A battle android guardian appears with mechanical plating ready to fold into another mode. kneels briefly as if receiving a command sequence. The scene is set in a ruined highway overpass, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A scholarly mage turns toward the storm with a ruby chain as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>A horned demon hero appears with a battle belt full of charms and relics. looks over one shoulder, alert for a second attack. The scene is set in a plaza of shattered statues and smoke, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. looks over one shoulder, alert for a second attack.</v>
+        <v>A mythic defender forged from every genre takes shape with a ruby blade as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>A glamorous demon queen appears with chunky retro panels in primary colors. lets sparks drift from her fingers without looking down. The scene is set in a shattered ballroom with broken chandeliers, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. lets sparks drift from her fingers without looking down.</v>
+        <v>An ember-eyed avenger breaks through the haze with a ruby pouch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>A cosmic tyrant appears with hands wrapped in crackling violet energy. waits without expression, which makes the threat worse. The scene is set in a cathedral of empty space, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. waits without expression, which makes the threat worse.</v>
+        <v>A moonlit temptress stands with dangerous grace with a ruby ring as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>A spiky-haired martial artist appears with a focused stare and wind whipping the hair upward. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a cliff edge above a storm sea, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A dimensional conqueror bends the sky with a ruby torch as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>A transforming robot knight appears with heavy shoulders shaped with anime clarity. turns the head just enough to suggest a human presence inside. The scene is set in a moonbase platform under floodlights, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. turns the head just enough to suggest a human presence inside.</v>
+        <v>A blue-flame combatant looks ready to leap with a ruby tablet as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>A hell-born guardian appears with a blade-hand forged from living fire. stands guard with one arm outstretched as if holding back a riot. The scene is set in a firelit dockyard full of black water, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. holds position with the stillness of a veteran.</v>
+        <v>A future war protector drops from the sky with a ruby key as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>A succubus antihero appears with a narrow waist and luminous mechanical limbs. stands with one hip angled, half invitation and half warning. The scene is set in a hangar full of red warning lights, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. stands poised like a queen deciding who may live.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a ruby mask as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>A void emperor appears with a chest core shining like a dying star. hovers above the scene like a sentence already carried out. The scene is set in a shattered asteroid throne hall, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. carries the stillness of a final boss before the last phase.</v>
+        <v>A mountain-raised berserker crouches low with a ruby idol as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>A supercharged fighter appears with a body built for speed and sudden impact. holds a stance that feels like the start of a new transformation. The scene is set in a ruined training hall, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>An arcane prodigy gathers light between the fingers with a ruby chalice as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>A chrome battle guardian appears with a body built from clean angular geometry. stands mid-transformation while plates shift and locks release. The scene is set in a drydock beside a stormy sea, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. locks into a battle form that looks ready for the final charge.</v>
+        <v>A last-boss guardian steps into the center of the scene with a ruby quartz as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>A volcanic avenger appears with a cloak stitched from soot-colored cloth. turns at three-quarters view while sparks climb the armor. The scene is set in a narrow canyon of apartment towers, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. steps forward through ash without breaking eye contact.</v>
+        <v>A horned guardian enters from the smoke with a opal lantern as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>A horned battle sorceress appears with a faceplate that opens into a calm human stare. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a neon alley reflecting rain on the pavement, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. spreads her wings as though she owns the air around her.</v>
+        <v>A glamorous demon queen poses without apology with a opal crown as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>A star-eating monarch appears with armor plated with sharp comet-like fins. stands perfectly still while debris orbits around him. The scene is set in a nebula storm full of lightning, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. rests one hand on a throne made of shattered moons.</v>
+        <v>A cosmic tyrant floats above the wreckage with a opal dagger as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>A gravity-breaking warrior appears with gloves wrapped in crackling energy bands. raises both hands in disciplined preparation for a special move. The scene is set in a forest clearing with torn banners, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A spiky-haired fighter surges into the shot with a opal banner as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>A vehicle-shaped mech hero appears with warning lights blinking across the torso. kneels briefly as if receiving a command sequence. The scene is set in a maintenance tunnel under a fortress, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a opal compass as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>A bat-winged vigilante appears with black obsidian armor with ember seams. leans into the wind as if the whole skyline is listening. The scene is set in a ruined chapel with torn banners, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A pale swordswoman stands in the rain with a opal mirror as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>A chrome guardian heroine appears with curved horns, violet eyes, and a jeweled corset of armor. holds still in a pose that feels expensive and lethal. The scene is set in a moonlit bridge over dark water, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A barbarian champion charges forward with a opal sigil as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>A dimensional conqueror appears with a crown of broken rings and black armor that drinks in starlight. raises a hand and makes the horizon feel smaller. The scene is set in a ruined observatory on a distant planet, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. stands perfectly still while debris orbits around him.</v>
+        <v>A wizard opens a glowing spellbook with a opal helm as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>A disciplined combat prodigy appears with an orange training suit and a bright electric aura. keeps his chin high as the aura swells around him. The scene is set in a rooftop under a violet lightning storm, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. raises both hands in disciplined preparation for a special move.</v>
+        <v>A final fusion champion stands in impossible balance with a opal orb as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>A towering machine duelist appears with silver armor panels and blue optics. braces in a landing pose with dust kicking outward. The scene is set in a shattered landing strip, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. kneels briefly as if receiving a command sequence.</v>
+        <v>A demon-born rescuer plants his feet with a opal chain as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>A red-skinned protector appears with a torn cape over scarred stone skin. holds position with the stillness of a veteran. The scene is set in a glassy intersection after a meteor strike, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. raises a fist to summon flame around the knuckles.</v>
+        <v>A horned enchantress steps into the frame with a opal blade as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>A machine-bodied temptress appears with translucent wings and clawed gloves. stands poised like a queen deciding who may live. The scene is set in a crystal crypt under a low ceiling of smoke, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A void emperor commands the frame with a opal pouch as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>A black-hole despot appears with purple lightning crawling over heavy metal plates. carries the stillness of a final boss before the last phase. The scene is set in a dark portal above a city, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. turns slightly as if the entire sky belongs to him.</v>
+        <v>A power-charged martial artist braces for impact with a opal ring as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>A tournament legend appears with silver hair, a torn gi, and sparks on the shoulders. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a canyon lined with fallen statues, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A chrome battle guardian shifts into combat form with a opal torch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>A future war protector appears with visible transformation seams and a reactor chest. locks into a battle form that looks ready for the final charge. The scene is set in a rusted factory floor, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. opens a chest panel to reveal a glowing core.</v>
+        <v>A scarred hunter moves through the ruins with a opal tablet as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>A cursed city sentinel appears with heavy gauntlets and a glowing chest sigil. plants a sword into the pavement like a promise. The scene is set in a stairway descending into red fog, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. looks over one shoulder, alert for a second attack.</v>
+        <v>A fur-clad warrior bellows in the open air with a opal key as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>A neon succubus pilot appears with polished white plating with bright blue optics. balances a weapon with theatrical ease. The scene is set in a vault of ancient machine parts, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. lets sparks drift from her fingers without looking down.</v>
+        <v>A battle mage lifts a hand and the air bends with a opal mask as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>A comet warlord appears with a cape shaped like a collapsing nebula. extends both arms as if pulling planets into place. The scene is set in a field of fragments from lost civilizations, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. waits without expression, which makes the threat worse.</v>
+        <v>An ultimate crossover hero fills the frame with a opal idol as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>A blue-flame brawler appears with a clenched fist surrounded by white light. leans forward, ready to cross the distance in one breath. The scene is set in a circular pit scarred by repeated battles, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A hell-forged vigilante turns toward the street with a opal chalice as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>A jet-form sentinel appears with blocky legs and sleek forearms. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a rooftop docking station, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. turns the head just enough to suggest a human presence inside.</v>
+        <v>A seductive antihero turns to face the viewer with a opal quartz as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>A smoke-wreathed champion appears with winged shoulder plates and clawed gloves. raises a fist to summon flame around the knuckles. The scene is set in a rain-slick alley lined with broken neon, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. holds position with the stillness of a veteran.</v>
+        <v>A star-eating monarch watches in silence with a bronze lantern as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>A black-winged war queen appears with a cockpit-like chest core and heavy machine joints. tilts her chin up as if challenging the viewer directly. The scene is set in a cathedral chamber lit by purple fire, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. stands poised like a queen deciding who may live.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a bronze crown as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>A galaxy breaker appears with a mask hiding every trace of mercy. turns slightly as if the entire sky belongs to him. The scene is set in a broken ring world, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. carries the stillness of a final boss before the last phase.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a bronze dagger as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>A sky-shattering combatant appears with boots planted wide on broken stone. settles into a low posture that promises a violent burst of speed. The scene is set in an arena floor split by shockwaves, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A grim blade carrier watches the tree line with a bronze banner as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>A tank-born champion appears with wing-like shoulder fins and bright thrusters. opens a chest panel to reveal a glowing core. The scene is set in a launch bay full of warning lights, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. locks into a battle form that looks ready for the final charge.</v>
+        <v>A savage axe fighter sets his stance with a bronze compass as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>A fire-eyed rescuer appears with a cracked helmet and blazing eyes. freezes for a beat before launching into motion. The scene is set in a collapsed overpass above a flooded street, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. steps forward through ash without breaking eye contact.</v>
+        <v>A spellcaster stands inside a circle of runes with a bronze mirror as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>A retro robot defender appears with smoke-colored hair and floating ember jewelry. turns just enough to show both beauty and threat. The scene is set in a black marble throne room, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. spreads her wings as though she owns the air around her.</v>
+        <v>A hybrid ruler of monsters and machines appears with a bronze sigil as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>An astral usurper appears with gravity ripples bending around the shoulders. walks forward through the void as though space is a corridor. The scene is set in the edge of a collapsing black hole, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. rests one hand on a throne made of shattered moons.</v>
+        <v>A black-winged defender walks into the light with a bronze helm as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>A dragon-aura hero appears with a face that stays calm for only a second. crouches as if the whole battle is a spring wound too tight. The scene is set in a mountain plateau under electric clouds, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a bronze orb as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>A stealth mech defender appears with a visor that opens like a cockpit canopy. spreads wing panels before taking off. The scene is set in a ruined highway overpass, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A galaxy breaker rises from the dark with a bronze chain as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>A shadow-cloaked defender appears with a broad chest wrapped in iron bands. steps forward through ash without breaking eye contact. The scene is set in a courthouse roof beneath a bruised sunset, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A tournament legend gathers force in silence with a bronze blade as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>A crimson inferno commander appears with a fitted bodysuit traced with circuit-like runes. spreads her wings as though she owns the air around her. The scene is set in a rooftop garden under a blood moon, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A towering machine duelist reconfigures its armor with a bronze pouch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>A moon-crowned ruler appears with an obsidian throne strapped to the back like a relic. rests one hand on a throne made of shattered moons. The scene is set in a dead moon covered in ice cliffs, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. stands perfectly still while debris orbits around him.</v>
+        <v>A battle-worn slayer pauses at the gate with a bronze ring as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>A hard-trained rival appears with a blue energy blaze rolling off the body. stands after impact as if the hit only sharpened his resolve. The scene is set in a desert plain with shattered pillars, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. raises both hands in disciplined preparation for a special move.</v>
+        <v>A tribal hero raises a weapon overhead with a bronze torch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>A winged machine paladin appears with mechanical plating ready to fold into another mode. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a smoke-filled hangar, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. kneels briefly as if receiving a command sequence.</v>
+        <v>A scholarly mage turns toward the storm with a bronze tablet as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>A crater-born hero appears with charcoal armor lit by molten cracks. keeps a low ready stance, built for protecting civilians first. The scene is set in a subway platform split by glowing cracks, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. raises a fist to summon flame around the knuckles.</v>
+        <v>A mythic defender forged from every genre takes shape with a bronze key as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>A sleek armored enchantress appears with a regal collar and black lacquered shoulder armor. keeps her hands relaxed even though the room feels dangerous. The scene is set in a foggy canal lined with lanterns, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. tilts her chin up as if challenging the viewer directly.</v>
+        <v>An ember-eyed avenger breaks through the haze with a bronze mask as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>A universe-devouring sovereign appears with glowing runes orbiting a towering silhouette. looks down at the world with pitiless patience. The scene is set in a starship graveyard, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. turns slightly as if the entire sky belongs to him.</v>
+        <v>A moonlit temptress stands with dangerous grace with a bronze idol as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>A power-surged champion appears with a sleeveless uniform shredded by battle. smiles briefly before tightening back into focus. The scene is set in a battlefield of smoke and broken stone, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A dimensional conqueror bends the sky with a bronze chalice as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>A battle android guardian appears with a sword mounted along the forearm. launches forward with sparks and motion blur trailing behind. The scene is set in a city street cracked by artillery fire, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. opens a chest panel to reveal a glowing core.</v>
+        <v>A blue-flame combatant looks ready to leap with a bronze quartz as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>A horned demon hero appears with a blade-hand forged from living fire. freezes for a beat before launching into motion. The scene is set in a narrow canyon of apartment towers, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. freezes for a beat before launching into motion.</v>
+        <v>A future war protector drops from the sky with a teal lantern as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>A glamorous demon queen appears with a narrow waist and luminous mechanical limbs. turns just enough to show both beauty and threat. The scene is set in a neon alley reflecting rain on the pavement, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. turns just enough to show both beauty and threat.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a teal crown as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>A cosmic tyrant appears with a chest core shining like a dying star. walks forward through the void as though space is a corridor. The scene is set in a nebula storm full of lightning, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. walks forward through the void as though space is a corridor.</v>
+        <v>A mountain-raised berserker crouches low with a teal dagger as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>A spiky-haired martial artist appears with a body built for speed and sudden impact. crouches as if the whole battle is a spring wound too tight. The scene is set in a forest clearing with torn banners, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>An arcane prodigy gathers light between the fingers with a teal banner as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>A transforming robot knight appears with a body built from clean angular geometry. spreads wing panels before taking off. The scene is set in a maintenance tunnel under a fortress, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. spreads wing panels before taking off.</v>
+        <v>A last-boss guardian steps into the center of the scene with a teal compass as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>A hell-born guardian appears with a cloak stitched from soot-colored cloth. steps forward through ash without breaking eye contact. The scene is set in a ruined chapel with torn banners, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A horned guardian enters from the smoke with a teal mirror as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>A succubus antihero appears with a faceplate that opens into a calm human stare. spreads her wings as though she owns the air around her. The scene is set in a moonlit bridge over dark water, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. stands with one hip angled, half invitation and half warning.</v>
+        <v>A glamorous demon queen poses without apology with a teal sigil as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>A void emperor appears with armor plated with sharp comet-like fins. rests one hand on a throne made of shattered moons. The scene is set in a ruined observatory on a distant planet, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. hovers above the scene like a sentence already carried out.</v>
+        <v>A cosmic tyrant floats above the wreckage with a teal helm as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>A supercharged fighter appears with gloves wrapped in crackling energy bands. stands after impact as if the hit only sharpened his resolve. The scene is set in a rooftop under a violet lightning storm, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. holds a stance that feels like the start of a new transformation.</v>
+        <v>A spiky-haired fighter surges into the shot with a teal orb as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>A chrome battle guardian appears with warning lights blinking across the torso. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a shattered landing strip, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. stands mid-transformation while plates shift and locks release.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a teal chain as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>A volcanic avenger appears with black obsidian armor with ember seams. keeps a low ready stance, built for protecting civilians first. The scene is set in a glassy intersection after a meteor strike, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. plants a sword into the pavement like a promise.</v>
+        <v>A pale swordswoman stands in the rain with a teal blade as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>A horned battle sorceress appears with curved horns, violet eyes, and a jeweled corset of armor. keeps her hands relaxed even though the room feels dangerous. The scene is set in a crystal crypt under a low ceiling of smoke, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. balances a weapon with theatrical ease.</v>
+        <v>A barbarian champion charges forward with a teal pouch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>A star-eating monarch appears with a crown of broken rings and black armor that drinks in starlight. looks down at the world with pitiless patience. The scene is set in a dark portal above a city, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. extends both arms as if pulling planets into place.</v>
+        <v>A wizard opens a glowing spellbook with a teal ring as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>A gravity-breaking warrior appears with an orange training suit and a bright electric aura. smiles briefly before tightening back into focus. The scene is set in a canyon lined with fallen statues, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. leans forward, ready to cross the distance in one breath.</v>
+        <v>A final fusion champion stands in impossible balance with a teal torch as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>A vehicle-shaped mech hero appears with silver armor panels and blue optics. launches forward with sparks and motion blur trailing behind. The scene is set in a rusted factory floor, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A demon-born rescuer plants his feet with a teal tablet as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>A bat-winged vigilante appears with a torn cape over scarred stone skin. looks over one shoulder, alert for a second attack. The scene is set in a stairway descending into red fog, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A horned enchantress steps into the frame with a teal key as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>A chrome guardian heroine appears with translucent wings and clawed gloves. lets sparks drift from her fingers without looking down. The scene is set in a vault of ancient machine parts, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>A void emperor commands the frame with a teal mask as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>A dimensional conqueror appears with purple lightning crawling over heavy metal plates. waits without expression, which makes the threat worse. The scene is set in a field of fragments from lost civilizations, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. looks down at the world with pitiless patience.</v>
+        <v>A power-charged martial artist braces for impact with a teal idol as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>A disciplined combat prodigy appears with silver hair, a torn gi, and sparks on the shoulders. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a circular pit scarred by repeated battles, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. smiles briefly before tightening back into focus.</v>
+        <v>A chrome battle guardian shifts into combat form with a teal chalice as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>A towering machine duelist appears with visible transformation seams and a reactor chest. turns the head just enough to suggest a human presence inside. The scene is set in a rooftop docking station, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A scarred hunter moves through the ruins with a teal quartz as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>A red-skinned protector appears with heavy gauntlets and a glowing chest sigil. stands guard with one arm outstretched as if holding back a riot. The scene is set in a rain-slick alley lined with broken neon, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. leans into the wind as if the whole skyline is listening.</v>
+        <v>A fur-clad warrior bellows in the open air with a indigo lantern as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>A machine-bodied temptress appears with polished white plating with bright blue optics. stands with one hip angled, half invitation and half warning. The scene is set in a cathedral chamber lit by purple fire, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. holds still in a pose that feels expensive and lethal.</v>
+        <v>A battle mage lifts a hand and the air bends with a indigo crown as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>A black-hole despot appears with a cape shaped like a collapsing nebula. hovers above the scene like a sentence already carried out. The scene is set in a broken ring world, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. raises a hand and makes the horizon feel smaller.</v>
+        <v>An ultimate crossover hero fills the frame with a indigo dagger as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>A tournament legend appears with a clenched fist surrounded by white light. holds a stance that feels like the start of a new transformation. The scene is set in an arena floor split by shockwaves, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. keeps his chin high as the aura swells around him.</v>
+        <v>A hell-forged vigilante turns toward the street with a indigo banner as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>A future war protector appears with blocky legs and sleek forearms. stands mid-transformation while plates shift and locks release. The scene is set in a launch bay full of warning lights, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. braces in a landing pose with dust kicking outward.</v>
+        <v>A seductive antihero turns to face the viewer with a indigo compass as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>A cursed city sentinel appears with winged shoulder plates and clawed gloves. turns at three-quarters view while sparks climb the armor. The scene is set in a collapsed overpass above a flooded street, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. freezes for a beat before launching into motion.</v>
+        <v>A star-eating monarch watches in silence with a indigo mirror as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>A neon succubus pilot appears with a cockpit-like chest core and heavy machine joints. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a black marble throne room, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. turns just enough to show both beauty and threat.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a indigo sigil as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>A comet warlord appears with a mask hiding every trace of mercy. stands perfectly still while debris orbits around him. The scene is set in the edge of a collapsing black hole, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. walks forward through the void as though space is a corridor.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a indigo helm as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>A blue-flame brawler appears with boots planted wide on broken stone. raises both hands in disciplined preparation for a special move. The scene is set in a mountain plateau under electric clouds, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. crouches as if the whole battle is a spring wound too tight.</v>
+        <v>A grim blade carrier watches the tree line with a indigo orb as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>A jet-form sentinel appears with wing-like shoulder fins and bright thrusters. kneels briefly as if receiving a command sequence. The scene is set in a ruined highway overpass, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. spreads wing panels before taking off.</v>
+        <v>A savage axe fighter sets his stance with a indigo chain as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>A smoke-wreathed champion appears with a cracked helmet and blazing eyes. leans into the wind as if the whole skyline is listening. The scene is set in a courthouse roof beneath a bruised sunset, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. stands guard with one arm outstretched as if holding back a riot.</v>
+        <v>A spellcaster stands inside a circle of runes with a indigo blade as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>A black-winged war queen appears with smoke-colored hair and floating ember jewelry. holds still in a pose that feels expensive and lethal. The scene is set in a rooftop garden under a blood moon, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. stands with one hip angled, half invitation and half warning.</v>
+        <v>A hybrid ruler of monsters and machines appears with a indigo pouch as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>A galaxy breaker appears with gravity ripples bending around the shoulders. raises a hand and makes the horizon feel smaller. The scene is set in a dead moon covered in ice cliffs, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. hovers above the scene like a sentence already carried out.</v>
+        <v>A black-winged defender walks into the light with a indigo ring as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>A sky-shattering combatant appears with a face that stays calm for only a second. keeps his chin high as the aura swells around him. The scene is set in a desert plain with shattered pillars, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. holds a stance that feels like the start of a new transformation.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a indigo torch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>A tank-born champion appears with a visor that opens like a cockpit canopy. braces in a landing pose with dust kicking outward. The scene is set in a smoke-filled hangar, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. stands mid-transformation while plates shift and locks release.</v>
+        <v>A galaxy breaker rises from the dark with a indigo tablet as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>A fire-eyed rescuer appears with a broad chest wrapped in iron bands. holds position with the stillness of a veteran. The scene is set in a subway platform split by glowing cracks, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. plants a sword into the pavement like a promise.</v>
+        <v>A tournament legend gathers force in silence with a indigo key as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>A retro robot defender appears with a fitted bodysuit traced with circuit-like runes. stands poised like a queen deciding who may live. The scene is set in a foggy canal lined with lanterns, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. balances a weapon with theatrical ease.</v>
+        <v>A towering machine duelist reconfigures its armor with a indigo mask as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>An astral usurper appears with an obsidian throne strapped to the back like a relic. carries the stillness of a final boss before the last phase. The scene is set in a starship graveyard, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. extends both arms as if pulling planets into place.</v>
+        <v>A battle-worn slayer pauses at the gate with a indigo idol as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>A dragon-aura hero appears with a blue energy blaze rolling off the body. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a battlefield of smoke and broken stone, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. leans forward, ready to cross the distance in one breath.</v>
+        <v>A tribal hero raises a weapon overhead with a indigo chalice as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>A stealth mech defender appears with mechanical plating ready to fold into another mode. locks into a battle form that looks ready for the final charge. The scene is set in a city street cracked by artillery fire, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. faces the viewer in a heroic stance that makes the machine feel alive.</v>
+        <v>A scholarly mage turns toward the storm with a indigo quartz as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>A shadow-cloaked defender appears with charcoal armor lit by molten cracks. plants a sword into the pavement like a promise. The scene is set in a plaza of shattered statues and smoke, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. keeps a low ready stance, built for protecting civilians first.</v>
+        <v>A mythic defender forged from every genre takes shape with a chalk lantern as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>A crimson inferno commander appears with a regal collar and black lacquered shoulder armor. balances a weapon with theatrical ease. The scene is set in a shattered ballroom with broken chandeliers, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. keeps her hands relaxed even though the room feels dangerous.</v>
+        <v>An ember-eyed avenger breaks through the haze with a chalk crown as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>A moon-crowned ruler appears with glowing runes orbiting a towering silhouette. extends both arms as if pulling planets into place. The scene is set in a cathedral of empty space, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. looks down at the world with pitiless patience.</v>
+        <v>A moonlit temptress stands with dangerous grace with a chalk dagger as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>A hard-trained rival appears with a sleeveless uniform shredded by battle. leans forward, ready to cross the distance in one breath. The scene is set in a cliff edge above a storm sea, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. smiles briefly before tightening back into focus.</v>
+        <v>A dimensional conqueror bends the sky with a chalk banner as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>A winged machine paladin appears with a sword mounted along the forearm. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a moonbase platform under floodlights, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. launches forward with sparks and motion blur trailing behind.</v>
+        <v>A blue-flame combatant looks ready to leap with a chalk compass as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>A crater-born hero appears with a battle belt full of charms and relics. raises a fist to summon flame around the knuckles. The scene is set in a firelit dockyard full of black water, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. leans into the wind as if the whole skyline is listening.</v>
+        <v>A future war protector drops from the sky with a chalk mirror as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>A sleek armored enchantress appears with chunky retro panels in primary colors. tilts her chin up as if challenging the viewer directly. The scene is set in a hangar full of red warning lights, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. holds still in a pose that feels expensive and lethal.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a chalk sigil as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>A universe-devouring sovereign appears with hands wrapped in crackling violet energy. turns slightly as if the entire sky belongs to him. The scene is set in a shattered asteroid throne hall, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. raises a hand and makes the horizon feel smaller.</v>
+        <v>A mountain-raised berserker crouches low with a chalk helm as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>A power-surged champion appears with a focused stare and wind whipping the hair upward. settles into a low posture that promises a violent burst of speed. The scene is set in a ruined training hall, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. keeps his chin high as the aura swells around him.</v>
+        <v>An arcane prodigy gathers light between the fingers with a chalk orb as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>A battle android guardian appears with heavy shoulders shaped with anime clarity. opens a chest panel to reveal a glowing core. The scene is set in a drydock beside a stormy sea, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. braces in a landing pose with dust kicking outward.</v>
+        <v>A last-boss guardian steps into the center of the scene with a chalk chain as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>A horned demon hero appears with a cloak stitched from soot-colored cloth. holds position with the stillness of a veteran. The scene is set in a glassy intersection after a meteor strike, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. holds position with the stillness of a veteran.</v>
+        <v>A horned guardian enters from the smoke with a chalk blade as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>A glamorous demon queen appears with a faceplate that opens into a calm human stare. stands poised like a queen deciding who may live. The scene is set in a crystal crypt under a low ceiling of smoke, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. stands poised like a queen deciding who may live.</v>
+        <v>A glamorous demon queen poses without apology with a chalk pouch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>A cosmic tyrant appears with armor plated with sharp comet-like fins. carries the stillness of a final boss before the last phase. The scene is set in a dark portal above a city, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. carries the stillness of a final boss before the last phase.</v>
+        <v>A cosmic tyrant floats above the wreckage with a chalk ring as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>A spiky-haired martial artist appears with gloves wrapped in crackling energy bands. faces the enemy with the confidence of someone who has never stopped training. The scene is set in a canyon lined with fallen statues, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A spiky-haired fighter surges into the shot with a chalk torch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="str">
-        <v>A transforming robot knight appears with warning lights blinking across the torso. locks into a battle form that looks ready for the final charge. The scene is set in a rusted factory floor, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. locks into a battle form that looks ready for the final charge.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a chalk tablet as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="str">
-        <v>A hell-born guardian appears with black obsidian armor with ember seams. plants a sword into the pavement like a promise. The scene is set in a stairway descending into red fog, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. steps forward through ash without breaking eye contact.</v>
+        <v>A pale swordswoman stands in the rain with a chalk key as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="str">
-        <v>A succubus antihero appears with curved horns, violet eyes, and a jeweled corset of armor. balances a weapon with theatrical ease. The scene is set in a vault of ancient machine parts, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. spreads her wings as though she owns the air around her.</v>
+        <v>A barbarian champion charges forward with a chalk mask as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="str">
-        <v>A void emperor appears with a crown of broken rings and black armor that drinks in starlight. extends both arms as if pulling planets into place. The scene is set in a field of fragments from lost civilizations, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. rests one hand on a throne made of shattered moons.</v>
+        <v>A wizard opens a glowing spellbook with a chalk idol as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="str">
-        <v>A supercharged fighter appears with an orange training suit and a bright electric aura. leans forward, ready to cross the distance in one breath. The scene is set in a circular pit scarred by repeated battles, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A final fusion champion stands in impossible balance with a chalk chalice as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="str">
-        <v>A chrome battle guardian appears with silver armor panels and blue optics. faces the viewer in a heroic stance that makes the machine feel alive. The scene is set in a rooftop docking station, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A demon-born rescuer plants his feet with a chalk quartz as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="str">
-        <v>A volcanic avenger appears with a torn cape over scarred stone skin. raises a fist to summon flame around the knuckles. The scene is set in a rain-slick alley lined with broken neon, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A horned enchantress steps into the frame with a smoke lantern as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="str">
-        <v>A horned battle sorceress appears with translucent wings and clawed gloves. tilts her chin up as if challenging the viewer directly. The scene is set in a cathedral chamber lit by purple fire, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>A void emperor commands the frame with a smoke crown as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="str">
-        <v>A star-eating monarch appears with purple lightning crawling over heavy metal plates. turns slightly as if the entire sky belongs to him. The scene is set in a broken ring world, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. stands perfectly still while debris orbits around him.</v>
+        <v>A power-charged martial artist braces for impact with a smoke dagger as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="str">
-        <v>A gravity-breaking warrior appears with silver hair, a torn gi, and sparks on the shoulders. settles into a low posture that promises a violent burst of speed. The scene is set in an arena floor split by shockwaves, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. raises both hands in disciplined preparation for a special move.</v>
+        <v>A chrome battle guardian shifts into combat form with a smoke banner as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="str">
-        <v>A vehicle-shaped mech hero appears with visible transformation seams and a reactor chest. opens a chest panel to reveal a glowing core. The scene is set in a launch bay full of warning lights, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. kneels briefly as if receiving a command sequence.</v>
+        <v>A scarred hunter moves through the ruins with a smoke compass as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="str">
-        <v>A bat-winged vigilante appears with heavy gauntlets and a glowing chest sigil. freezes for a beat before launching into motion. The scene is set in a collapsed overpass above a flooded street, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. raises a fist to summon flame around the knuckles.</v>
+        <v>A fur-clad warrior bellows in the open air with a smoke mirror as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="str">
-        <v>A chrome guardian heroine appears with polished white plating with bright blue optics. turns just enough to show both beauty and threat. The scene is set in a black marble throne room, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A battle mage lifts a hand and the air bends with a smoke sigil as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="str">
-        <v>A dimensional conqueror appears with a cape shaped like a collapsing nebula. walks forward through the void as though space is a corridor. The scene is set in the edge of a collapsing black hole, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. turns slightly as if the entire sky belongs to him.</v>
+        <v>An ultimate crossover hero fills the frame with a smoke helm as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="str">
-        <v>A disciplined combat prodigy appears with a clenched fist surrounded by white light. crouches as if the whole battle is a spring wound too tight. The scene is set in a mountain plateau under electric clouds, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. settles into a low posture that promises a violent burst of speed.</v>
+        <v>A hell-forged vigilante turns toward the street with a smoke orb as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="str">
-        <v>A towering machine duelist appears with blocky legs and sleek forearms. spreads wing panels before taking off. The scene is set in a ruined highway overpass, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. opens a chest panel to reveal a glowing core.</v>
+        <v>A seductive antihero turns to face the viewer with a smoke chain as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="str">
-        <v>A red-skinned protector appears with winged shoulder plates and clawed gloves. steps forward through ash without breaking eye contact. The scene is set in a courthouse roof beneath a bruised sunset, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. looks over one shoulder, alert for a second attack.</v>
+        <v>A star-eating monarch watches in silence with a smoke blade as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="str">
-        <v>A machine-bodied temptress appears with a cockpit-like chest core and heavy machine joints. spreads her wings as though she owns the air around her. The scene is set in a rooftop garden under a blood moon, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. lets sparks drift from her fingers without looking down.</v>
+        <v>A gravity-breaking warrior holds a perfect stance with a smoke pouch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="str">
-        <v>A black-hole despot appears with a mask hiding every trace of mercy. rests one hand on a throne made of shattered moons. The scene is set in a dead moon covered in ice cliffs, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. waits without expression, which makes the threat worse.</v>
+        <v>A vehicle-shaped mech hero unfolds midair with a smoke ring as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="str">
-        <v>A tournament legend appears with boots planted wide on broken stone. stands after impact as if the hit only sharpened his resolve. The scene is set in a desert plain with shattered pillars, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A grim blade carrier watches the tree line with a smoke torch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="str">
-        <v>A future war protector appears with wing-like shoulder fins and bright thrusters. holds a sword in one hand as the other arm reconfigures into a shield. The scene is set in a smoke-filled hangar, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. turns the head just enough to suggest a human presence inside.</v>
+        <v>A savage axe fighter sets his stance with a smoke tablet as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="str">
-        <v>A cursed city sentinel appears with a cracked helmet and blazing eyes. keeps a low ready stance, built for protecting civilians first. The scene is set in a subway platform split by glowing cracks, and The face should read as protective rather than cruel. The face should read as protective rather than cruel. holds position with the stillness of a veteran.</v>
+        <v>A spellcaster stands inside a circle of runes with a smoke key as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="str">
-        <v>A neon succubus pilot appears with smoke-colored hair and floating ember jewelry. keeps her hands relaxed even though the room feels dangerous. The scene is set in a foggy canal lined with lanterns, and The result should feel glamorous, dangerous, and instantly readable. The result should feel glamorous, dangerous, and instantly readable. stands poised like a queen deciding who may live.</v>
+        <v>A hybrid ruler of monsters and machines appears with a smoke mask as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="str">
-        <v>A comet warlord appears with gravity ripples bending around the shoulders. looks down at the world with pitiless patience. The scene is set in a starship graveyard, and The scale should feel immense and unnerving. The scale should feel immense and unnerving. carries the stillness of a final boss before the last phase.</v>
+        <v>A black-winged defender walks into the light with a smoke idol as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="str">
-        <v>A blue-flame brawler appears with a face that stays calm for only a second. smiles briefly before tightening back into focus. The scene is set in a battlefield of smoke and broken stone, and The energy should feel bright and cinematic. The energy should feel bright and cinematic. faces the enemy with the confidence of someone who has never stopped training.</v>
+        <v>A crimson-winged sorceress claims the spotlight with a smoke chalice as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="str">
-        <v>A jet-form sentinel appears with a visor that opens like a cockpit canopy. launches forward with sparks and motion blur trailing behind. The scene is set in a city street cracked by artillery fire, and The design must read cleanly as heroic machinery. The design must read cleanly as heroic machinery. locks into a battle form that looks ready for the final charge.</v>
+        <v>A galaxy breaker rises from the dark with a smoke quartz as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="str">
-        <v>A smoke-wreathed champion appears with a broad chest wrapped in iron bands. looks over one shoulder, alert for a second attack. The scene is set in a plaza of shattered statues and smoke, and The palette should lean to ember red, soot black, and old gold. The image should have the polish of a dramatic comic cover. steps forward through ash without breaking eye contact.</v>
+        <v>A tournament legend gathers force in silence with a sunlit lantern as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="str">
-        <v>A black-winged war queen appears with a fitted bodysuit traced with circuit-like runes. lets sparks drift from her fingers without looking down. The scene is set in a shattered ballroom with broken chandeliers, and The scene needs to balance seduction with mechanical precision. Treat the figure like the star of a dark fantasy poster. spreads her wings as though she owns the air around her.</v>
+        <v>A towering machine duelist reconfigures its armor with a sunlit crown as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="str">
-        <v>A galaxy breaker appears with an obsidian throne strapped to the back like a relic. waits without expression, which makes the threat worse. The scene is set in a cathedral of empty space, and The palette should lean to violet, steel, and ultraviolet glow. The villain should be calm, not frantic. rests one hand on a throne made of shattered moons.</v>
+        <v>A battle-worn slayer pauses at the gate with a sunlit dagger as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="str">
-        <v>A sky-shattering combatant appears with a blue energy blaze rolling off the body. looks calm enough to be dangerous, which makes the next strike feel bigger. The scene is set in a cliff edge above a storm sea, and The form should read like a legendary anime power-up. The scene should feel like the hero just unlocked a higher level. stands after impact as if the hit only sharpened his resolve.</v>
+        <v>A tribal hero raises a weapon overhead with a sunlit banner as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="str">
-        <v>A tank-born champion appears with mechanical plating ready to fold into another mode. turns the head just enough to suggest a human presence inside. The scene is set in a moonbase platform under floodlights, and The metal should catch highlights so it feels tangible. The image should look like a major mecha reveal. holds a sword in one hand as the other arm reconfigures into a shield.</v>
+        <v>A scholarly mage turns toward the storm with a sunlit compass as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="str">
-        <v>A fire-eyed rescuer appears with charcoal armor lit by molten cracks. stands guard with one arm outstretched as if holding back a riot. The scene is set in a firelit dockyard full of black water, and The silhouette needs to feel iconic from a distance. The palette should lean to ember red, soot black, and old gold. turns at three-quarters view while sparks climb the armor.</v>
+        <v>A mythic defender forged from every genre takes shape with a sunlit mirror as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="str">
-        <v>A retro robot defender appears with a regal collar and black lacquered shoulder armor. stands with one hip angled, half invitation and half warning. The scene is set in a hangar full of red warning lights, and The lighting should sharpen the horns, metal, and cheekbones. The scene needs to balance seduction with mechanical precision. moves in a slow, deliberate step that makes everyone else feel slower.</v>
+        <v>An ember-eyed avenger breaks through the haze with a sunlit sigil as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="str">
-        <v>An astral usurper appears with glowing runes orbiting a towering silhouette. hovers above the scene like a sentence already carried out. The scene is set in a shattered asteroid throne hall, and A soft pastel contrast element can make the menace feel surreal. The palette should lean to violet, steel, and ultraviolet glow. stands perfectly still while debris orbits around him.</v>
+        <v>A moonlit temptress stands with dangerous grace with a sunlit helm as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="str">
-        <v>A dragon-aura hero appears with a sleeveless uniform shredded by battle. holds a stance that feels like the start of a new transformation. The scene is set in a ruined training hall, and The body language must sell speed, discipline, and raw force. The form should read like a legendary anime power-up. raises both hands in disciplined preparation for a special move.</v>
+        <v>A dimensional conqueror bends the sky with a sunlit orb as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="str">
-        <v>A stealth mech defender appears with a sword mounted along the forearm. stands mid-transformation while plates shift and locks release. The scene is set in a drydock beside a stormy sea, and A human pilot can add emotion without stealing focus. The metal should catch highlights so it feels tangible. kneels briefly as if receiving a command sequence.</v>
+        <v>A blue-flame combatant looks ready to leap with a sunlit chain as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="str">
-        <v>A shadow-cloaked defender appears with a battle belt full of charms and relics. turns at three-quarters view while sparks climb the armor. The scene is set in a narrow canyon of apartment towers, and The image should have the polish of a dramatic comic cover. Keep the sense of danger, but make the heroism unmistakable. raises a fist to summon flame around the knuckles.</v>
+        <v>A future war protector drops from the sky with a sunlit blade as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="str">
-        <v>A crimson inferno commander appears with chunky retro panels in primary colors. moves in a slow, deliberate step that makes everyone else feel slower. The scene is set in a neon alley reflecting rain on the pavement, and Treat the figure like the star of a dark fantasy poster. The character should feel like she could lead an army or ruin one. tilts her chin up as if challenging the viewer directly.</v>
+        <v>A haunted duelist grips a weapon taller than she is with a sunlit pouch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="str">
-        <v>A moon-crowned ruler appears with hands wrapped in crackling violet energy. stands perfectly still while debris orbits around him. The scene is set in a nebula storm full of lightning, and The villain should be calm, not frantic. The final image should feel like the climax of a space opera. turns slightly as if the entire sky belongs to him.</v>
+        <v>A mountain-raised berserker crouches low with a sunlit ring as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="str">
-        <v>A hard-trained rival appears with a focused stare and wind whipping the hair upward. raises both hands in disciplined preparation for a special move. The scene is set in a forest clearing with torn banners, and The scene should feel like the hero just unlocked a higher level. Use debris and motion to make the impact believable. settles into a low posture that promises a violent burst of speed.</v>
+        <v>An arcane prodigy gathers light between the fingers with a sunlit torch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="str">
-        <v>A winged machine paladin appears with heavy shoulders shaped with anime clarity. kneels briefly as if receiving a command sequence. The scene is set in a maintenance tunnel under a fortress, and The image should look like a major mecha reveal. The silhouette needs a memorable weapon shape. opens a chest panel to reveal a glowing core.</v>
+        <v>A last-boss guardian steps into the center of the scene with a sunlit tablet as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="str">
-        <v>A crater-born hero appears with a blade-hand forged from living fire. leans into the wind as if the whole skyline is listening. The scene is set in a ruined chapel with torn banners, and Keep the sense of danger, but make the heroism unmistakable. The silhouette needs to feel iconic from a distance. looks over one shoulder, alert for a second attack.</v>
+        <v>A horned guardian enters from the smoke with a sunlit key as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="str">
-        <v>A sleek armored enchantress appears with a narrow waist and luminous mechanical limbs. holds still in a pose that feels expensive and lethal. The scene is set in a moonlit bridge over dark water, and The character should feel like she could lead an army or ruin one. The lighting should sharpen the horns, metal, and cheekbones. lets sparks drift from her fingers without looking down.</v>
+        <v>A glamorous demon queen poses without apology with a sunlit mask as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="str">
-        <v>A universe-devouring sovereign appears with a chest core shining like a dying star. raises a hand and makes the horizon feel smaller. The scene is set in a ruined observatory on a distant planet, and The final image should feel like the climax of a space opera. A soft pastel contrast element can make the menace feel surreal. waits without expression, which makes the threat worse.</v>
+        <v>A cosmic tyrant floats above the wreckage with a sunlit idol as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="str">
-        <v>A power-surged champion appears with a body built for speed and sudden impact. keeps his chin high as the aura swells around him. The scene is set in a rooftop under a violet lightning storm, and Use debris and motion to make the impact believable. The body language must sell speed, discipline, and raw force. looks calm enough to be dangerous, which makes the next strike feel bigger.</v>
+        <v>A spiky-haired fighter surges into the shot with a sunlit chalice as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="str">
-        <v>A battle android guardian appears with a body built from clean angular geometry. braces in a landing pose with dust kicking outward. The scene is set in a shattered landing strip, and The silhouette needs a memorable weapon shape. A human pilot can add emotion without stealing focus. turns the head just enough to suggest a human presence inside.</v>
+        <v>A transforming robot knight lands in a burst of sparks with a sunlit quartz as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild prompts with authored visual direction
</commit_message>
<xml_diff>
--- a/Infinity_Forge_Prompts_Master.xlsx
+++ b/Infinity_Forge_Prompts_Master.xlsx
@@ -398,2505 +398,2508 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A500"/>
+  <cols>
+    <col min="1" max="1" width="110.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>A horned guardian enters from the smoke with a amber lantern as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>A glamorous demon queen poses without apology with a amber crown as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a amber dagger as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>A spiky-haired fighter surges into the shot with a amber banner as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a amber compass as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>A pale swordswoman stands in the rain with a amber mirror as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>A barbarian champion charges forward with a amber sigil as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>A wizard opens a glowing spellbook with a amber helm as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>A final fusion champion stands in impossible balance with a amber orb as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>A demon-born rescuer plants his feet with a amber chain as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In vaults beneath a dead cathedral, the subject kneels in a pool of candle wax and presses the prop against a sealed crypt door, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. low three-quarter view, candlelight cutting upward across the face. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>A horned enchantress steps into the frame with a amber blade as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>A void emperor commands the frame with a amber pouch as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>A power-charged martial artist braces for impact with a amber ring as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>A chrome battle guardian shifts into combat form with a amber torch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>A scarred hunter moves through the ruins with a amber tablet as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>A fur-clad warrior bellows in the open air with a amber key as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>A battle mage lifts a hand and the air bends with a amber mask as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>An ultimate crossover hero fills the frame with a amber idol as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>A hell-forged vigilante turns toward the street with a amber chalice as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>A seductive antihero turns to face the viewer with a amber quartz as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a flooded subway platform, the subject balances on a toppled train while reaching toward a child-sized emergency beacon, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. long-lens view through rain-streaked glass, green station lights behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>A star-eating monarch watches in silence with a crimson lantern as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a crimson crown as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a crimson dagger as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>A grim blade carrier watches the tree line with a crimson banner as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>A savage axe fighter sets his stance with a crimson compass as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>A spellcaster stands inside a circle of runes with a crimson mirror as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a crimson sigil as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>A black-winged defender walks into the light with a crimson helm as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a crimson orb as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>A galaxy breaker rises from the dark with a crimson chain as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a red desert at eclipse, the subject drives one foot into the sand and catches a falling obelisk against one shoulder, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. wide low angle, the eclipsed sun forming a hard rim around the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>A tournament legend gathers force in silence with a crimson blade as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>A towering machine duelist reconfigures its armor with a crimson pouch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>A battle-worn slayer pauses at the gate with a crimson ring as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>A tribal hero raises a weapon overhead with a crimson torch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>A scholarly mage turns toward the storm with a crimson tablet as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>A mythic defender forged from every genre takes shape with a crimson key as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a crimson mask as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a crimson idol as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>A dimensional conqueror bends the sky with a crimson chalice as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>A blue-flame combatant looks ready to leap with a crimson quartz as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a winter harbor, the subject slides across black ice with the prop extended toward an incoming wave, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. side-on tracking composition, pale dawn and spray frozen in motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>A future war protector drops from the sky with a cerulean lantern as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a cerulean crown as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>A mountain-raised berserker crouches low with a cerulean dagger as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a cerulean banner as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a cerulean compass as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>A horned guardian enters from the smoke with a cerulean mirror as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>A glamorous demon queen poses without apology with a cerulean sigil as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a cerulean helm as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>A spiky-haired fighter surges into the shot with a cerulean orb as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a cerulean chain as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a greenhouse overtaken by jungle, the subject cuts through hanging vines while luminous moths scatter from the blade, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. intimate shoulder-height framing, humid backlight and layered leaves. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>A pale swordswoman stands in the rain with a cerulean blade as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>A barbarian champion charges forward with a cerulean pouch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>A wizard opens a glowing spellbook with a cerulean ring as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>A final fusion champion stands in impossible balance with a cerulean torch as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>A demon-born rescuer plants his feet with a cerulean tablet as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>A horned enchantress steps into the frame with a cerulean key as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>A void emperor commands the frame with a cerulean mask as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>A power-charged martial artist braces for impact with a cerulean idol as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>A chrome battle guardian shifts into combat form with a cerulean chalice as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>A scarred hunter moves through the ruins with a cerulean quartz as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a ruined observatory, the subject stands on the rotating dome as broken constellations project across the armor, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. vertiginous overhead composition, cold starlight and brass reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>A fur-clad warrior bellows in the open air with a ashen lantern as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>A battle mage lifts a hand and the air bends with a ashen crown as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>An ultimate crossover hero fills the frame with a ashen dagger as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>A hell-forged vigilante turns toward the street with a ashen banner as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>A seductive antihero turns to face the viewer with a ashen compass as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>A star-eating monarch watches in silence with a ashen mirror as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a ashen sigil as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a ashen helm as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>A grim blade carrier watches the tree line with a ashen orb as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>A savage axe fighter sets his stance with a ashen chain as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a crowded night market, the subject turns sideways between startled vendors, protecting a stall with the prop, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. street-level documentary angle, lanterns and steam creating depth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>A spellcaster stands inside a circle of runes with a ashen blade as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a ashen pouch as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>A black-winged defender walks into the light with a ashen ring as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a ashen torch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>A galaxy breaker rises from the dark with a ashen tablet as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>A tournament legend gathers force in silence with a ashen key as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>A towering machine duelist reconfigures its armor with a ashen mask as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>A battle-worn slayer pauses at the gate with a ashen idol as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>A tribal hero raises a weapon overhead with a ashen chalice as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>A scholarly mage turns toward the storm with a ashen quartz as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a canyon during a sandstorm, the subject plants the prop as an anchor while fabric and dust whip violently around the body, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. compressed telephoto portrait, only the eyes and silhouette remain sharp. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>A mythic defender forged from every genre takes shape with a emerald lantern as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a emerald crown as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a emerald dagger as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>A dimensional conqueror bends the sky with a emerald banner as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>A blue-flame combatant looks ready to leap with a emerald compass as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>A future war protector drops from the sky with a emerald mirror as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a emerald sigil as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>A mountain-raised berserker crouches low with a emerald helm as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a emerald orb as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a emerald chain as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a black-water marsh, the subject wades knee-deep through reeds while a submerged creature circles behind, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. quiet frontal composition, moonlit ripples leading toward the subject. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>A horned guardian enters from the smoke with a emerald blade as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>A glamorous demon queen poses without apology with a emerald pouch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a emerald ring as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>A spiky-haired fighter surges into the shot with a emerald torch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a emerald tablet as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>A pale swordswoman stands in the rain with a emerald key as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>A barbarian champion charges forward with a emerald mask as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>A wizard opens a glowing spellbook with a emerald idol as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>A final fusion champion stands in impossible balance with a emerald chalice as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>A demon-born rescuer plants his feet with a emerald quartz as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a shattered bridge above clouds, the subject leaps across a gap with one knee raised and the prop trailing behind, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. dynamic diagonal frame, clouds below and hard sunlight on the edge. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>A horned enchantress steps into the frame with a violet lantern as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>A void emperor commands the frame with a violet crown as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>A power-charged martial artist braces for impact with a violet dagger as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>A chrome battle guardian shifts into combat form with a violet banner as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>A scarred hunter moves through the ruins with a violet compass as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>A fur-clad warrior bellows in the open air with a violet mirror as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>A battle mage lifts a hand and the air bends with a violet sigil as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>An ultimate crossover hero fills the frame with a violet helm as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>A hell-forged vigilante turns toward the street with a violet orb as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>A seductive antihero turns to face the viewer with a violet chain as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In an abandoned carnival, the subject stands beneath a dead ferris wheel while gripping the prop like a warning, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. centered symmetrical frame, faded bulbs and wet asphalt reflections. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>A star-eating monarch watches in silence with a violet blade as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a violet pouch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a violet ring as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>A grim blade carrier watches the tree line with a violet torch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>A savage axe fighter sets his stance with a violet tablet as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>A spellcaster stands inside a circle of runes with a violet key as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a violet mask as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>A black-winged defender walks into the light with a violet idol as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a violet chalice as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>A galaxy breaker rises from the dark with a violet quartz as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a volcanic forge, the subject swings the prop through a shower of sparks as unfinished armor hangs nearby, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. close action crop, orange furnace light against deep blue shadow. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>A tournament legend gathers force in silence with a golden lantern as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>A towering machine duelist reconfigures its armor with a golden crown as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>A battle-worn slayer pauses at the gate with a golden dagger as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>A tribal hero raises a weapon overhead with a golden banner as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>A scholarly mage turns toward the storm with a golden compass as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>A mythic defender forged from every genre takes shape with a golden mirror as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a golden sigil as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a golden helm as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>A dimensional conqueror bends the sky with a golden orb as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>A blue-flame combatant looks ready to leap with a golden chain as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a palace hallway filled with mirrors, the subject rests the prop on one shoulder while every reflection shows a different stance, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. long corridor perspective, repeating reflections used as the composition. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>A future war protector drops from the sky with a golden blade as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a golden pouch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>A mountain-raised berserker crouches low with a golden ring as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a golden torch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a golden tablet as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>A horned guardian enters from the smoke with a golden key as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>A glamorous demon queen poses without apology with a golden mask as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a golden idol as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>A spiky-haired fighter surges into the shot with a golden chalice as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a golden quartz as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a moonlit rice terrace, the subject steps between flooded fields with the prop held low and ready, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. high wide view, silver water planes and a small human silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>A pale swordswoman stands in the rain with a silver lantern as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>A barbarian champion charges forward with a silver crown as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>A wizard opens a glowing spellbook with a silver dagger as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>A final fusion champion stands in impossible balance with a silver banner as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>A demon-born rescuer plants his feet with a silver compass as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>A horned enchantress steps into the frame with a silver mirror as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>A void emperor commands the frame with a silver sigil as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>A power-charged martial artist braces for impact with a silver helm as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>A chrome battle guardian shifts into combat form with a silver orb as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>A scarred hunter moves through the ruins with a silver chain as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a storm-battered lighthouse stairwell, the subject climbs upward two steps at a time with the prop catching the rotating beam, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. spiral composition from above, white beam slicing through salt mist. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>A fur-clad warrior bellows in the open air with a silver blade as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>A battle mage lifts a hand and the air bends with a silver pouch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>An ultimate crossover hero fills the frame with a silver ring as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>A hell-forged vigilante turns toward the street with a silver torch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>A seductive antihero turns to face the viewer with a silver tablet as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>A star-eating monarch watches in silence with a silver key as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a silver mask as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a silver idol as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>A grim blade carrier watches the tree line with a silver chalice as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>A savage axe fighter sets his stance with a silver quartz as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a neon repair district, the subject crouches beside a sparking machine and uses the prop to redirect current, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. angled close-up, cyan signage reflected on metal and wet pavement. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>A spellcaster stands inside a circle of runes with a cobalt lantern as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a cobalt crown as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>A black-winged defender walks into the light with a cobalt dagger as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a cobalt banner as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>A galaxy breaker rises from the dark with a cobalt compass as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>A tournament legend gathers force in silence with a cobalt mirror as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>A towering machine duelist reconfigures its armor with a cobalt sigil as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>A battle-worn slayer pauses at the gate with a cobalt helm as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>A tribal hero raises a weapon overhead with a cobalt orb as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>A scholarly mage turns toward the storm with a cobalt chain as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a salt flat after rain, the subject walks toward the camera with the prop lowered, mirrored sky doubling the figure, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. minimalist full-body frame, horizon near the upper third. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>A mythic defender forged from every genre takes shape with a cobalt blade as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a cobalt pouch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a cobalt ring as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>A dimensional conqueror bends the sky with a cobalt torch as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>A blue-flame combatant looks ready to leap with a cobalt tablet as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>A future war protector drops from the sky with a cobalt key as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a cobalt mask as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>A mountain-raised berserker crouches low with a cobalt idol as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a cobalt chalice as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a cobalt quartz as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a library where the books are floating, the subject reaches through drifting pages to seize the prop while loose papers orbit the body, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. gentle upward view, warm reading lamps against a dark ceiling. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>A horned guardian enters from the smoke with a obsidian lantern as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>A glamorous demon queen poses without apology with a obsidian crown as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a obsidian dagger as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>A spiky-haired fighter surges into the shot with a obsidian banner as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a obsidian compass as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>A pale swordswoman stands in the rain with a obsidian mirror as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>A barbarian champion charges forward with a obsidian sigil as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>A wizard opens a glowing spellbook with a obsidian helm as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>A final fusion champion stands in impossible balance with a obsidian orb as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>A demon-born rescuer plants his feet with a obsidian chain as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In an ancient battlefield at sunrise, the subject drags the prop from the earth and looks toward distant banners, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. wide environmental portrait, long shadows and copper haze. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>A horned enchantress steps into the frame with a obsidian blade as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>A void emperor commands the frame with a obsidian pouch as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>A power-charged martial artist braces for impact with a obsidian ring as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>A chrome battle guardian shifts into combat form with a obsidian torch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>A scarred hunter moves through the ruins with a obsidian tablet as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>A fur-clad warrior bellows in the open air with a obsidian key as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>A battle mage lifts a hand and the air bends with a obsidian mask as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>An ultimate crossover hero fills the frame with a obsidian idol as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>A hell-forged vigilante turns toward the street with a obsidian chalice as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>A seductive antihero turns to face the viewer with a obsidian quartz as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a narrow apartment balcony, the subject sits on the railing with the prop across the knees, watching the city wake, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. quiet 85mm portrait, layered windows and muted morning color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>A star-eating monarch watches in silence with a ivory lantern as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a ivory crown as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a ivory dagger as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>A grim blade carrier watches the tree line with a ivory banner as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>A savage axe fighter sets his stance with a ivory compass as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>A spellcaster stands inside a circle of runes with a ivory mirror as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a ivory sigil as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>A black-winged defender walks into the light with a ivory helm as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a ivory orb as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>A galaxy breaker rises from the dark with a ivory chain as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a glacier crevasse, the subject hangs from a rope with one hand and hooks the prop over a ledge with the other, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. vertical top-down view, blue ice walls framing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>A tournament legend gathers force in silence with a ivory blade as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>A towering machine duelist reconfigures its armor with a ivory pouch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>A battle-worn slayer pauses at the gate with a ivory ring as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>A tribal hero raises a weapon overhead with a ivory torch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>A scholarly mage turns toward the storm with a ivory tablet as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>A mythic defender forged from every genre takes shape with a ivory key as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a ivory mask as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a ivory idol as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>A dimensional conqueror bends the sky with a ivory chalice as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>A blue-flame combatant looks ready to leap with a ivory quartz as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a ballroom after a supernatural blackout, the subject dances backward across the floor while keeping the prop aimed at an unseen threat, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. wide lens at waist height, emergency candles reflected in polished wood. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>A future war protector drops from the sky with a scarlet lantern as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a scarlet crown as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>A mountain-raised berserker crouches low with a scarlet dagger as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a scarlet banner as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a scarlet compass as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>A horned guardian enters from the smoke with a scarlet mirror as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>A glamorous demon queen poses without apology with a scarlet sigil as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a scarlet helm as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>A spiky-haired fighter surges into the shot with a scarlet orb as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a scarlet chain as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a floating market above the clouds, the subject steps from one wooden boat to another while the prop balances overhead, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. high-angle travel frame, sails and cloud layers giving scale. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>A pale swordswoman stands in the rain with a scarlet blade as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>A barbarian champion charges forward with a scarlet pouch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>A wizard opens a glowing spellbook with a scarlet ring as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>A final fusion champion stands in impossible balance with a scarlet torch as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>A demon-born rescuer plants his feet with a scarlet tablet as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>A horned enchantress steps into the frame with a scarlet key as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>A void emperor commands the frame with a scarlet mask as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>A power-charged martial artist braces for impact with a scarlet idol as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>A chrome battle guardian shifts into combat form with a scarlet chalice as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>A scarred hunter moves through the ruins with a scarlet quartz as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a subterranean river, the subject stands on a narrow stone fin as bioluminescent water rushes around the boots, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. long exposure feeling, cool glow outlining the posture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>A fur-clad warrior bellows in the open air with a jade lantern as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>A battle mage lifts a hand and the air bends with a jade crown as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>An ultimate crossover hero fills the frame with a jade dagger as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>A hell-forged vigilante turns toward the street with a jade banner as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>A seductive antihero turns to face the viewer with a jade compass as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>A star-eating monarch watches in silence with a jade mirror as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a jade sigil as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a jade helm as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>A grim blade carrier watches the tree line with a jade orb as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>A savage axe fighter sets his stance with a jade chain as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a battlefield made from toppled statues, the subject leans against a broken marble face and reloads or resets the prop with deliberate calm, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. medium shot, dust shafts and monumental fragments behind. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>A spellcaster stands inside a circle of runes with a jade blade as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a jade pouch as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>A black-winged defender walks into the light with a jade ring as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a jade torch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>A galaxy breaker rises from the dark with a jade tablet as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>A tournament legend gathers force in silence with a jade key as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>A towering machine duelist reconfigures its armor with a jade mask as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>A battle-worn slayer pauses at the gate with a jade idol as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>A tribal hero raises a weapon overhead with a jade chalice as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>A scholarly mage turns toward the storm with a jade quartz as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a rain-soaked rooftop garden, the subject kneels among tomato vines while the prop reflects a distant lightning strike, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. close portrait, storm sky and red fruit as color accents. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>A mythic defender forged from every genre takes shape with a saffron lantern as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a saffron crown as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a saffron dagger as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>A dimensional conqueror bends the sky with a saffron banner as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>A blue-flame combatant looks ready to leap with a saffron compass as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>A future war protector drops from the sky with a saffron mirror as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a saffron sigil as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>A mountain-raised berserker crouches low with a saffron helm as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a saffron orb as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a saffron chain as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a brass airship deck, the subject braces against the rail while the prop points toward another vessel in the fog, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. three-quarter rear view, cables and propellers creating framing lines. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>A horned guardian enters from the smoke with a saffron blade as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>A glamorous demon queen poses without apology with a saffron pouch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a saffron ring as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>A spiky-haired fighter surges into the shot with a saffron torch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a saffron tablet as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>A pale swordswoman stands in the rain with a saffron key as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>A barbarian champion charges forward with a saffron mask as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>A wizard opens a glowing spellbook with a saffron idol as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>A final fusion champion stands in impossible balance with a saffron chalice as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>A demon-born rescuer plants his feet with a saffron quartz as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a haunted school gymnasium, the subject stands at center court as chalk diagrams ignite beneath the feet, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. high overhead composition, geometric floor markings and stark shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>A horned enchantress steps into the frame with a pearl lantern as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>A void emperor commands the frame with a pearl crown as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>A power-charged martial artist braces for impact with a pearl dagger as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="str">
-        <v>A chrome battle guardian shifts into combat form with a pearl banner as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>A scarred hunter moves through the ruins with a pearl compass as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>A fur-clad warrior bellows in the open air with a pearl mirror as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>A battle mage lifts a hand and the air bends with a pearl sigil as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>An ultimate crossover hero fills the frame with a pearl helm as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>A hell-forged vigilante turns toward the street with a pearl orb as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>A seductive antihero turns to face the viewer with a pearl chain as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a canyon of giant red flowers, the subject pushes through petals taller than the body, using the prop to part a path, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. low macro-like perspective, pollen glowing in afternoon light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>A star-eating monarch watches in silence with a pearl blade as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a pearl pouch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a pearl ring as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>A grim blade carrier watches the tree line with a pearl torch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>A savage axe fighter sets his stance with a pearl tablet as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>A spellcaster stands inside a circle of runes with a pearl key as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a pearl mask as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>A black-winged defender walks into the light with a pearl idol as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a pearl chalice as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="str">
-        <v>A galaxy breaker rises from the dark with a pearl quartz as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a silent spaceport, the subject waits beside a sealed gate with the prop tucked under one arm and a ticket in the other, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. wide cinematic frame, terminal architecture dwarfing the figure. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="str">
-        <v>A tournament legend gathers force in silence with a onyx lantern as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>A towering machine duelist reconfigures its armor with a onyx crown as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>A battle-worn slayer pauses at the gate with a onyx dagger as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
-        <v>A tribal hero raises a weapon overhead with a onyx banner as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="str">
-        <v>A scholarly mage turns toward the storm with a onyx compass as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="str">
-        <v>A mythic defender forged from every genre takes shape with a onyx mirror as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a onyx sigil as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a onyx helm as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>A dimensional conqueror bends the sky with a onyx orb as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>A blue-flame combatant looks ready to leap with a onyx chain as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a clockwork chapel, the subject pulls a brass lever while gears rotate behind the shoulders, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. profile composition, hard shafts of light and intricate mechanical texture. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>A future war protector drops from the sky with a onyx blade as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a onyx pouch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>A mountain-raised berserker crouches low with a onyx ring as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a onyx torch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a onyx tablet as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>A horned guardian enters from the smoke with a onyx key as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>A glamorous demon queen poses without apology with a onyx mask as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a onyx idol as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>A spiky-haired fighter surges into the shot with a onyx chalice as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a onyx quartz as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a coastal cliff at blue hour, the subject casts the prop into the wind as if testing its weight before a duel, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. distant silhouette, sea spray and violet horizon. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
-        <v>A pale swordswoman stands in the rain with a moss lantern as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="str">
-        <v>A barbarian champion charges forward with a moss crown as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>A wizard opens a glowing spellbook with a moss dagger as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>A final fusion champion stands in impossible balance with a moss banner as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>A demon-born rescuer plants his feet with a moss compass as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="str">
-        <v>A horned enchantress steps into the frame with a moss mirror as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="str">
-        <v>A void emperor commands the frame with a moss sigil as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="str">
-        <v>A power-charged martial artist braces for impact with a moss helm as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="str">
-        <v>A chrome battle guardian shifts into combat form with a moss orb as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="str">
-        <v>A scarred hunter moves through the ruins with a moss chain as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a shattered moon temple, the subject floats inches above the floor while the prop points at a rotating lunar map, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. upward-looking composition, fragments suspended in weightlessness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>A fur-clad warrior bellows in the open air with a moss blade as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>A battle mage lifts a hand and the air bends with a moss pouch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>An ultimate crossover hero fills the frame with a moss ring as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>A hell-forged vigilante turns toward the street with a moss torch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>A seductive antihero turns to face the viewer with a moss tablet as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>A star-eating monarch watches in silence with a moss key as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a moss mask as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a moss idol as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>A grim blade carrier watches the tree line with a moss chalice as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>A savage axe fighter sets his stance with a moss quartz as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a crowded underground arena, the subject steps through a ring of spectators with the prop resting against the shoulder, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. circular composition, faces and banners forming a living frame. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>A spellcaster stands inside a circle of runes with a ruby lantern as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a ruby crown as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>A black-winged defender walks into the light with a ruby dagger as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a ruby banner as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>A galaxy breaker rises from the dark with a ruby compass as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>A tournament legend gathers force in silence with a ruby mirror as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>A towering machine duelist reconfigures its armor with a ruby sigil as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>A battle-worn slayer pauses at the gate with a ruby helm as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>A tribal hero raises a weapon overhead with a ruby orb as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>A scholarly mage turns toward the storm with a ruby chain as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a forest of petrified trees, the subject touches one stone trunk and watches cracks of light travel toward the prop, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. quiet side profile, narrow shafts of gold between gray forms. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>A mythic defender forged from every genre takes shape with a ruby blade as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a ruby pouch as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a ruby ring as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>A dimensional conqueror bends the sky with a ruby torch as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>A blue-flame combatant looks ready to leap with a ruby tablet as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>A future war protector drops from the sky with a ruby key as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a ruby mask as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>A mountain-raised berserker crouches low with a ruby idol as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a ruby chalice as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a ruby quartz as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a flooded museum, the subject swims beneath a submerged dinosaur skeleton while clutching the prop to the chest, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. underwater wide angle, wavering light and floating labels. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>A horned guardian enters from the smoke with a opal lantern as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>A glamorous demon queen poses without apology with a opal crown as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a opal dagger as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>A spiky-haired fighter surges into the shot with a opal banner as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a opal compass as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>A pale swordswoman stands in the rain with a opal mirror as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>A barbarian champion charges forward with a opal sigil as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>A wizard opens a glowing spellbook with a opal helm as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>A final fusion champion stands in impossible balance with a opal orb as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>A demon-born rescuer plants his feet with a opal chain as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a rooftop during the first snow, the subject plants the prop beside a small rooftop garden and shields a flame with both hands, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. intimate medium frame, soft flakes against charcoal city shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>A horned enchantress steps into the frame with a opal blade as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>A void emperor commands the frame with a opal pouch as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>A power-charged martial artist braces for impact with a opal ring as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>A chrome battle guardian shifts into combat form with a opal torch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>A scarred hunter moves through the ruins with a opal tablet as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>A fur-clad warrior bellows in the open air with a opal key as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>A battle mage lifts a hand and the air bends with a opal mask as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>An ultimate crossover hero fills the frame with a opal idol as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>A hell-forged vigilante turns toward the street with a opal chalice as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>A seductive antihero turns to face the viewer with a opal quartz as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a canyon bridge made of bones, the subject crosses cautiously with the prop held behind the body to counterbalance each step, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. dramatic vanishing point, warm sunset through the ribs. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>A star-eating monarch watches in silence with a bronze lantern as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a bronze crown as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a bronze dagger as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>A grim blade carrier watches the tree line with a bronze banner as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>A savage axe fighter sets his stance with a bronze compass as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>A spellcaster stands inside a circle of runes with a bronze mirror as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a bronze sigil as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>A black-winged defender walks into the light with a bronze helm as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a bronze orb as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>A galaxy breaker rises from the dark with a bronze chain as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a ruined theater stage, the subject takes a final bow while the prop remains hidden behind the curtain, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. front-facing stage composition, empty seats fading into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>A tournament legend gathers force in silence with a bronze blade as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>A towering machine duelist reconfigures its armor with a bronze pouch as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>A battle-worn slayer pauses at the gate with a bronze ring as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>A tribal hero raises a weapon overhead with a bronze torch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>A scholarly mage turns toward the storm with a bronze tablet as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>A mythic defender forged from every genre takes shape with a bronze key as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a bronze mask as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a bronze idol as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>A dimensional conqueror bends the sky with a bronze chalice as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>A blue-flame combatant looks ready to leap with a bronze quartz as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a field of blue lightning, the subject walks between grounded bolts with the prop held vertically like a lightning rod, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. wide negative-space frame, electric branches defining the silhouette. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>A future war protector drops from the sky with a teal lantern as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a teal crown as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>A mountain-raised berserker crouches low with a teal dagger as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a teal banner as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a teal compass as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>A horned guardian enters from the smoke with a teal mirror as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>A glamorous demon queen poses without apology with a teal sigil as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a teal helm as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>A spiky-haired fighter surges into the shot with a teal orb as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a teal chain as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a palace kitchen during an evacuation, the subject lifts a heavy table to reveal a hidden passage while cooks flee around the body, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. handheld-feeling low angle, flour dust and warm copper pans. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>A pale swordswoman stands in the rain with a teal blade as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>A barbarian champion charges forward with a teal pouch as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>A wizard opens a glowing spellbook with a teal ring as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>A final fusion champion stands in impossible balance with a teal torch as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>A demon-born rescuer plants his feet with a teal tablet as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>A horned enchantress steps into the frame with a teal key as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>A void emperor commands the frame with a teal mask as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>A power-charged martial artist braces for impact with a teal idol as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>A chrome battle guardian shifts into combat form with a teal chalice as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>A scarred hunter moves through the ruins with a teal quartz as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a desert caravan at night, the subject sits beside a lantern and repairs the prop with a tiny tool kit, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. close campfire portrait, patterned blankets and distant dunes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>A fur-clad warrior bellows in the open air with a indigo lantern as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>A battle mage lifts a hand and the air bends with a indigo crown as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>An ultimate crossover hero fills the frame with a indigo dagger as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>A hell-forged vigilante turns toward the street with a indigo banner as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>A seductive antihero turns to face the viewer with a indigo compass as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>A star-eating monarch watches in silence with a indigo mirror as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a indigo sigil as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a indigo helm as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>A grim blade carrier watches the tree line with a indigo orb as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>A savage axe fighter sets his stance with a indigo chain as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a waterfall cave, the subject emerges from the curtain of water with the prop dripping and ready, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. frontal heroic reveal, mist softening the cave mouth. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>A spellcaster stands inside a circle of runes with a indigo blade as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a indigo pouch as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>A black-winged defender walks into the light with a indigo ring as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a indigo torch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>A galaxy breaker rises from the dark with a indigo tablet as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>A tournament legend gathers force in silence with a indigo key as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>A towering machine duelist reconfigures its armor with a indigo mask as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>A battle-worn slayer pauses at the gate with a indigo idol as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>A tribal hero raises a weapon overhead with a indigo chalice as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>A scholarly mage turns toward the storm with a indigo quartz as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a city intersection frozen in time, the subject walks through suspended rain drops while every nearby clock points to a different hour, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. wide street perspective, crisp subject against stopped motion. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>A mythic defender forged from every genre takes shape with a chalk lantern as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a chalk crown as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a chalk dagger as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>A dimensional conqueror bends the sky with a chalk banner as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>A blue-flame combatant looks ready to leap with a chalk compass as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>A future war protector drops from the sky with a chalk mirror as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a chalk sigil as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>A mountain-raised berserker crouches low with a chalk helm as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a chalk orb as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a chalk chain as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a field of giant sleeping beasts, the subject tiptoes between massive ribs with the prop held close to avoid waking them, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. high aerial view, tiny figure surrounded by organic shapes. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>A horned guardian enters from the smoke with a chalk blade as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>A glamorous demon queen poses without apology with a chalk pouch as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a chalk ring as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>A spiky-haired fighter surges into the shot with a chalk torch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a chalk tablet as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="str">
-        <v>A pale swordswoman stands in the rain with a chalk key as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Place her in a ruined village with wet stone and one lonely lantern. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="str">
-        <v>A barbarian champion charges forward with a chalk mask as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Let the battlefield stretch behind him with banners, smoke, and broken shields. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="str">
-        <v>A wizard opens a glowing spellbook with a chalk idol as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The image should feel like a high-energy anime spell duel with clear geometry. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="str">
-        <v>A final fusion champion stands in impossible balance with a chalk chalice as a focal prop. Every part of the costume should feel deliberate and story-rich. Use a huge readable silhouette so the design still works at thumbnail size. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="str">
-        <v>A demon-born rescuer plants his feet with a chalk quartz as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Set him against a flooded avenue and let the firelight reflect from the water. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a mountain shrine in heavy fog, the subject rings a ceremonial bell with the prop while prayer ribbons stream behind, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. minimal centered composition, red ribbons as the only saturated color. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="str">
-        <v>A horned enchantress steps into the frame with a smoke lantern as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. The scene works best in a black marble hall with smoke drifting along the floor. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="str">
-        <v>A void emperor commands the frame with a smoke crown as a focal prop. The pose should be so controlled that the air seems to orbit around him. The atmosphere should feel like a space opera collapsing into silence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="str">
-        <v>A power-charged martial artist braces for impact with a smoke dagger as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The background should look like the setup to a decisive finishing move. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="str">
-        <v>A chrome battle guardian shifts into combat form with a smoke banner as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Set the machine in a hangar lit by warning strips and rising steam. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="str">
-        <v>A scarred hunter moves through the ruins with a smoke compass as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. A broken chapel or chapel aisle will intensify the gothic mood. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="str">
-        <v>A fur-clad warrior bellows in the open air with a smoke mirror as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The mood should feel wild, heroic, and like a legend told around a fire. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="str">
-        <v>A battle mage lifts a hand and the air bends with a smoke sigil as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Use luminous blues, golds, and whites to separate the spellwork from the background. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="str">
-        <v>An ultimate crossover hero fills the frame with a smoke helm as a focal prop. Every part of the costume should feel deliberate and story-rich. The final result should feel like the biggest battle imaginable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="str">
-        <v>A hell-forged vigilante turns toward the street with a smoke orb as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Place the scene on a collapsed rooftop so the silhouette cuts cleanly against the sky. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="str">
-        <v>A seductive antihero turns to face the viewer with a smoke chain as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. A shattered ballroom or moonlit balcony would make the pose feel even more dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In an underground train tunnel, the subject plants a hand against the wall as the prop illuminates a fresh trail of symbols, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. narrow perspective, repeating lights pulling the eye into darkness. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="str">
-        <v>A star-eating monarch watches in silence with a smoke blade as a focal prop. The pose should be so controlled that the air seems to orbit around him. Use cold highlights and violent purple glow to separate him from the void. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="str">
-        <v>A gravity-breaking warrior holds a perfect stance with a smoke pouch as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Put him in a shattered arena with dust hanging in the air. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="str">
-        <v>A vehicle-shaped mech hero unfolds midair with a smoke ring as a focal prop. The overall silhouette must be heroic and easy to identify in motion. A ruined freeway or launch pad would give the transformation a strong sense of scale. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="str">
-        <v>A grim blade carrier watches the tree line with a smoke torch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The scene should feel like a western adult cartoon with dark fantasy and horror influence. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="str">
-        <v>A savage axe fighter sets his stance with a smoke tablet as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Use earthy browns, iron gray, and fire orange to make the world feel harsh. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="str">
-        <v>A spellcaster stands inside a circle of runes with a smoke key as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. The final piece should feel intelligent, dramatic, and visually crisp. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="str">
-        <v>A hybrid ruler of monsters and machines appears with a smoke mask as a focal prop. Every part of the costume should feel deliberate and story-rich. Set the figure in a storm of shattered stone and drifting debris. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="str">
-        <v>A black-winged defender walks into the light with a smoke idol as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. A cracked courthouse or subway entry would make the scene feel grounded and dramatic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="str">
-        <v>A crimson-winged sorceress claims the spotlight with a smoke chalice as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Use a rich fantasy palette so the image feels expensive, eerie, and memorable. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="str">
-        <v>A galaxy breaker rises from the dark with a smoke quartz as a focal prop. The pose should be so controlled that the air seems to orbit around him. Place him near a broken ring world so the scale feels enormous. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a palace roof during a festival, the subject perches on a tiled ridge and watches fireworks bloom behind the prop, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. telephoto portrait, layered fireworks and glowing paper lanterns. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="str">
-        <v>A tournament legend gathers force in silence with a sunlit lantern as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. A mountain plateau under electric clouds would make the aura feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="str">
-        <v>A towering machine duelist reconfigures its armor with a sunlit crown as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Let sparks, cables, and smoke trail behind the figure as it lands. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="str">
-        <v>A battle-worn slayer pauses at the gate with a sunlit dagger as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. Use sparse color, hard shadows, and a lonely atmosphere. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="str">
-        <v>A tribal hero raises a weapon overhead with a sunlit banner as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. The final image should be primal, direct, and easy to understand at a glance. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="str">
-        <v>A scholarly mage turns toward the storm with a sunlit compass as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. Place the figure in a library ruin with floating pages and dust motes. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="str">
-        <v>A mythic defender forged from every genre takes shape with a sunlit mirror as a focal prop. Every part of the costume should feel deliberate and story-rich. Let city ruins, starfire, and fantasy relics collide in one coherent composition. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="str">
-        <v>An ember-eyed avenger breaks through the haze with a sunlit sigil as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. The background should feel like a world where one strong protector still matters. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="str">
-        <v>A moonlit temptress stands with dangerous grace with a sunlit helm as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Set her in a throne room lit by violet fire and reflected candlelight. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="str">
-        <v>A dimensional conqueror bends the sky with a sunlit orb as a focal prop. The pose should be so controlled that the air seems to orbit around him. A black hole or shattered moon would make the scene feel truly cosmic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="str">
-        <v>A blue-flame combatant looks ready to leap with a sunlit chain as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. The scene should have enough debris and motion cues to imply a huge clash just happened. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a frozen battlefield at noon, the subject raises the prop overhead while old weapons protrude from the snow around the boots, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. crisp high-contrast full-body shot, white ground and cobalt shadows. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="str">
-        <v>A future war protector drops from the sky with a sunlit blade as a focal prop. The overall silhouette must be heroic and easy to identify in motion. The scene should feel like the moment before a big mecha reveal in an animated series. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Hand-authored fantasy character concept, depict male infernal guardian: a tall, broad-shouldered man with charcoal skin, two swept-back obsidian horns, ember-orange eyes, a braided black beard, cracked basalt armor over a soot-stained red tunic, and a chain-wrapped greatshield. a demon-born protector who turns his body into a barricade for strangers. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a shield rimmed with living coal clearly readable. Keep the torso square and both feet planted, with the near hand protecting the chest. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="str">
-        <v>A haunted duelist grips a weapon taller than she is with a sunlit pouch as a focal prop. She looks exhausted in the way only a veteran monster hunter can look exhausted. The image should read as mature, somber, and cinematic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Cinematic production design portrait, depict female mutant sky sentinel: a muscular woman with cobalt skin, short white hair, silver irises, a star-shaped mark across one cheek, a fitted red-and-gold flight suit, translucent energy wings, and heavy gauntlets. a weather-tested aerial rescuer who treats the storm as an opponent. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a broken satellite panel used as a shield clearly readable. Twist the hips away from the threat while the rear foot skids for traction and the free hand reaches back. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="str">
-        <v>A mountain-raised berserker crouches low with a sunlit ring as a focal prop. Fur, leather, bone charms, and scarred skin should tell a story of hard living. Set the character in a torchlit war camp with rough wooden defenses. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Detailed key art for an original animated feature, depict male demon warlock: a lean man with russet skin, one curled horn, pale ritual scars across his chest, a shaved head with a long topknot, layered violet robes, a bone clasp, and ink-black fingers. a patient occult strategist whose spells are built from contracts and geometry. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a brass astrolabe leaking blue fire clearly readable. Use a compact crouch with one knee nearly touching the ground, shoulders angled toward the next escape route. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="str">
-        <v>An arcane prodigy gathers light between the fingers with a sunlit torch as a focal prop. Magic effects should be visible and purposeful rather than decorative haze. A stormy battlefield with glowing circles in the sky would make the magic feel huge. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Editorial creature-and-hero illustration, depict female succubus duelist: a poised woman with wine-red skin, swept ram horns, long silver hair, gold eyes, batlike wings folded behind a black velvet coat, high boots, and a narrow rapier. a smiling underworld negotiator who wins every argument at sword point. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a mirror-bright rapier catching the moon clearly readable. Show a long diagonal stride, the leading shoulder low and the trailing garment describing the movement. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="str">
-        <v>A last-boss guardian steps into the center of the scene with a sunlit tablet as a focal prop. Every part of the costume should feel deliberate and story-rich. The image should feel like demons, robots, anime fighters, and dark fantasy all colliding at once. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>High-end game splash art, depict male gobot salvage knight: a compact orange-and-teal robotic man assembled from chunky panels, exposed pistons, a square visor, tire-like heels, riveted shoulder plates, and a fold-out welding torch. a tireless machine rescuer built to repair wrecks under impossible pressure. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a magnetic crane arm loaded with salvaged parts clearly readable. Give the figure a guarded side stance, elbows bent and weight resting on the back leg. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="str">
-        <v>A horned guardian enters from the smoke with a sunlit key as a focal prop. He carries a protective tension, like someone who has chosen duty over comfort. Use a city ruin, broken neon, and drifting ash so the figure feels like a last defender. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Painterly graphic novel cover, depict female cosmic tyrant: a towering woman with porcelain skin, a smooth violet crown fused to her skull, black star-shaped eyes, a segmented white battle mantle, floating gold rings, and six silent gravity orbs. an immaculate conqueror who regards planets as pieces on a game board. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a miniature blue planet suspended between two fingers clearly readable. Capture a suspended instant with the body folded slightly forward and the prop pulled close to the ribs. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="str">
-        <v>A glamorous demon queen poses without apology with a sunlit mask as a focal prop. The costume should feel luxurious, sharp, and fully functional at the same time. Place her on a rain-wet rooftop with city lights stretching behind her. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Practical-effects fantasy film still, depict male martial energy fighter: a compact, heavily muscled man with spiky black hair, dark eyes, orange sleeveless training clothes, blue wrist wraps, worn boots, and a torn sash snapping in the wind. a cheerful tournament fighter whose concentrated force distorts the landscape. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a glowing sphere of compressed energy clearly readable. Let the subject lean into the environment, one hand braced against a surface while the other controls the prop. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="str">
-        <v>A cosmic tyrant floats above the wreckage with a sunlit idol as a focal prop. The pose should be so controlled that the air seems to orbit around him. Let tiny pastel bear-like guardians drift in the distance for a surreal contrast. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Moody science-fantasy character study, depict female transforming robot knight: a tall crimson-and-silver robotic woman with a sharp helmet crest, luminous cyan optics, articulated wings, tank-tread calves, a shield folded into her forearm, and a sword made from a vehicle door. a disciplined machine commander who changes configuration mid-strike. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a half-transformed shield locking into place clearly readable. Use an open, off-balance recovery pose, one heel lifted and the head turned toward something outside frame. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="str">
-        <v>A spiky-haired fighter surges into the shot with a sunlit chalice as a focal prop. The stance should be simple but iconic, like a frame you would remember instantly. Use bright energy trails and hard shadows so the figure feels alive and kinetic. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Premium collectible art direction, depict male pale monster slayer: a wiry pale man with shoulder-length ash hair, a vertical scar over one eye, layered leather armor, a weathered gray cloak, fingerless gloves, and a huge claymore balanced across one shoulder. a quiet hunter who studies monstrous anatomy before committing to a single devastating cut. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a blood-dark greatsword with a chipped fuller clearly readable. Frame a deliberate pause after exertion: shoulders rising from breath, knees soft, weapon lowered but ready. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="str">
-        <v>A transforming robot knight lands in a burst of sparks with a sunlit quartz as a focal prop. The overall silhouette must be heroic and easy to identify in motion. Keep the composition sharp, dramatic, and highly legible. The final image should feel like a hand-directed, high-end image prompt rather than a recycled template.</v>
+        <v>Story-rich animation cels translated into finished illustration, depict female armored spellblade: a dark-skinned woman with copper braids, amber eyes, a blue hood pushed behind her neck, lacquered scale armor, a rune-etched longsword, and a leather spellbook chained to her belt. a battlefield scholar who uses precise footwork instead of theatrical gestures. In a workshop after an explosion, the subject stands amid hanging cables and scattered tools, holding the prop away from a smoking crater, with a spellbook opening in the wind beside her blade clearly readable. Show a sharp directional turn, coat, hair, cables, or wings lagging behind the rotation of the head. off-center composition, amber dust and sharp rim light. Show believable anatomy or engineered joints, tactile surface wear, deliberate hand placement, and a distinct silhouette; build the lighting from the environment so the face, costume materials, and action remain legible. No text, logos, watermark, or generic stock pose.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>